<commit_message>
feat: suporte BTS/COLLO e expansao do layout widescreen com tabela espacosa
</commit_message>
<xml_diff>
--- a/public/templates/NDD-bts.xlsx
+++ b/public/templates/NDD-bts.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8338DE85-A1F8-4E0F-8097-E0985C9A0151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE33401-3373-4F09-9E21-7FD26C2FC753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1199,6 +1199,306 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1289,310 +1589,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2030,121 +2030,121 @@
   <sheetData>
     <row r="1" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="173" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="79" t="s">
+      <c r="B2" s="174"/>
+      <c r="C2" s="174"/>
+      <c r="D2" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="79"/>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="79"/>
-      <c r="P2" s="80"/>
-      <c r="Q2" s="85"/>
-      <c r="R2" s="86"/>
-      <c r="S2" s="87"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
+      <c r="L2" s="179"/>
+      <c r="M2" s="179"/>
+      <c r="N2" s="179"/>
+      <c r="O2" s="179"/>
+      <c r="P2" s="180"/>
+      <c r="Q2" s="185"/>
+      <c r="R2" s="186"/>
+      <c r="S2" s="187"/>
       <c r="U2" t="str">
         <f t="array" aca="1" ref="U2" ca="1">CELL("nome.arquivo")</f>
-        <v>C:\Users\ValtemirJunior\Downloads\NDD - Forge\public\templates\[NDD-padrao.xlsx]NDD</v>
+        <v>C:\Users\ValtemirJunior\Downloads\NDD - Forge\public\templates\[NDD-bts.xlsx]NDD</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="75"/>
-      <c r="B3" s="76"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="81"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="88"/>
-      <c r="R3" s="89"/>
-      <c r="S3" s="90"/>
+      <c r="A3" s="175"/>
+      <c r="B3" s="176"/>
+      <c r="C3" s="176"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
+      <c r="H3" s="181"/>
+      <c r="I3" s="181"/>
+      <c r="J3" s="181"/>
+      <c r="K3" s="181"/>
+      <c r="L3" s="181"/>
+      <c r="M3" s="181"/>
+      <c r="N3" s="181"/>
+      <c r="O3" s="181"/>
+      <c r="P3" s="182"/>
+      <c r="Q3" s="188"/>
+      <c r="R3" s="189"/>
+      <c r="S3" s="190"/>
       <c r="U3" t="e">
         <f ca="1">MID(U2,FIND("WINITY_",U2)+7,FIND("_MT",U2)-FIND("WINITY_",U2)-7)</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="81"/>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
-      <c r="G4" s="81"/>
-      <c r="H4" s="81"/>
-      <c r="I4" s="81"/>
-      <c r="J4" s="81"/>
-      <c r="K4" s="81"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="81"/>
-      <c r="N4" s="81"/>
-      <c r="O4" s="81"/>
-      <c r="P4" s="82"/>
-      <c r="Q4" s="88"/>
-      <c r="R4" s="89"/>
-      <c r="S4" s="90"/>
+      <c r="A4" s="175"/>
+      <c r="B4" s="176"/>
+      <c r="C4" s="176"/>
+      <c r="D4" s="181"/>
+      <c r="E4" s="181"/>
+      <c r="F4" s="181"/>
+      <c r="G4" s="181"/>
+      <c r="H4" s="181"/>
+      <c r="I4" s="181"/>
+      <c r="J4" s="181"/>
+      <c r="K4" s="181"/>
+      <c r="L4" s="181"/>
+      <c r="M4" s="181"/>
+      <c r="N4" s="181"/>
+      <c r="O4" s="181"/>
+      <c r="P4" s="182"/>
+      <c r="Q4" s="188"/>
+      <c r="R4" s="189"/>
+      <c r="S4" s="190"/>
       <c r="U4" t="e">
         <f ca="1">TRIM(U3)</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5" s="77"/>
-      <c r="B5" s="78"/>
-      <c r="C5" s="78"/>
-      <c r="D5" s="83"/>
-      <c r="E5" s="83"/>
-      <c r="F5" s="83"/>
-      <c r="G5" s="83"/>
-      <c r="H5" s="83"/>
-      <c r="I5" s="83"/>
-      <c r="J5" s="83"/>
-      <c r="K5" s="83"/>
-      <c r="L5" s="83"/>
-      <c r="M5" s="83"/>
-      <c r="N5" s="83"/>
-      <c r="O5" s="83"/>
-      <c r="P5" s="84"/>
-      <c r="Q5" s="91"/>
-      <c r="R5" s="92"/>
-      <c r="S5" s="93"/>
+      <c r="A5" s="177"/>
+      <c r="B5" s="178"/>
+      <c r="C5" s="178"/>
+      <c r="D5" s="183"/>
+      <c r="E5" s="183"/>
+      <c r="F5" s="183"/>
+      <c r="G5" s="183"/>
+      <c r="H5" s="183"/>
+      <c r="I5" s="183"/>
+      <c r="J5" s="183"/>
+      <c r="K5" s="183"/>
+      <c r="L5" s="183"/>
+      <c r="M5" s="183"/>
+      <c r="N5" s="183"/>
+      <c r="O5" s="183"/>
+      <c r="P5" s="184"/>
+      <c r="Q5" s="191"/>
+      <c r="R5" s="192"/>
+      <c r="S5" s="193"/>
     </row>
     <row r="6" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="94" t="s">
+      <c r="A6" s="194" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="95"/>
-      <c r="C6" s="95"/>
+      <c r="B6" s="195"/>
+      <c r="C6" s="195"/>
       <c r="D6" s="2">
         <f ca="1">TODAY()</f>
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E6" s="3"/>
-      <c r="F6" s="96"/>
-      <c r="G6" s="96"/>
-      <c r="H6" s="96"/>
-      <c r="I6" s="96"/>
-      <c r="J6" s="96"/>
+      <c r="F6" s="196"/>
+      <c r="G6" s="196"/>
+      <c r="H6" s="196"/>
+      <c r="I6" s="196"/>
+      <c r="J6" s="196"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
@@ -2156,21 +2156,21 @@
       <c r="S6" s="5"/>
     </row>
     <row r="7" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="97" t="s">
+      <c r="A7" s="197" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="98"/>
-      <c r="C7" s="98"/>
+      <c r="B7" s="198"/>
+      <c r="C7" s="198"/>
       <c r="D7" s="2" t="e">
         <f>_xlfn.XLOOKUP(C9,#REF!,#REF!,"")</f>
         <v>#REF!</v>
       </c>
       <c r="E7" s="3"/>
-      <c r="F7" s="99"/>
-      <c r="G7" s="99"/>
-      <c r="H7" s="99"/>
-      <c r="I7" s="99"/>
-      <c r="J7" s="99"/>
+      <c r="F7" s="199"/>
+      <c r="G7" s="199"/>
+      <c r="H7" s="199"/>
+      <c r="I7" s="199"/>
+      <c r="J7" s="199"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
@@ -2182,74 +2182,74 @@
       <c r="S7" s="7"/>
     </row>
     <row r="8" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="100" t="s">
+      <c r="A8" s="200" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="101"/>
-      <c r="C8" s="101"/>
-      <c r="D8" s="101"/>
-      <c r="E8" s="101"/>
-      <c r="F8" s="101"/>
-      <c r="G8" s="101"/>
-      <c r="H8" s="101"/>
-      <c r="I8" s="101"/>
-      <c r="J8" s="101"/>
-      <c r="K8" s="101"/>
-      <c r="L8" s="101"/>
-      <c r="M8" s="101"/>
-      <c r="N8" s="101"/>
-      <c r="O8" s="101"/>
-      <c r="P8" s="101"/>
-      <c r="Q8" s="101"/>
-      <c r="R8" s="101"/>
-      <c r="S8" s="102"/>
+      <c r="B8" s="201"/>
+      <c r="C8" s="201"/>
+      <c r="D8" s="201"/>
+      <c r="E8" s="201"/>
+      <c r="F8" s="201"/>
+      <c r="G8" s="201"/>
+      <c r="H8" s="201"/>
+      <c r="I8" s="201"/>
+      <c r="J8" s="201"/>
+      <c r="K8" s="201"/>
+      <c r="L8" s="201"/>
+      <c r="M8" s="201"/>
+      <c r="N8" s="201"/>
+      <c r="O8" s="201"/>
+      <c r="P8" s="201"/>
+      <c r="Q8" s="201"/>
+      <c r="R8" s="201"/>
+      <c r="S8" s="202"/>
     </row>
     <row r="9" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="103" t="s">
+      <c r="A9" s="155" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="104"/>
-      <c r="C9" s="105"/>
-      <c r="D9" s="106"/>
+      <c r="B9" s="165"/>
+      <c r="C9" s="203"/>
+      <c r="D9" s="156"/>
       <c r="E9" s="9"/>
       <c r="F9" s="10"/>
-      <c r="G9" s="107" t="s">
+      <c r="G9" s="167" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="106"/>
-      <c r="I9" s="108"/>
-      <c r="J9" s="108"/>
-      <c r="K9" s="108"/>
-      <c r="L9" s="109"/>
-      <c r="M9" s="110" t="s">
+      <c r="H9" s="156"/>
+      <c r="I9" s="158"/>
+      <c r="J9" s="158"/>
+      <c r="K9" s="158"/>
+      <c r="L9" s="166"/>
+      <c r="M9" s="168" t="s">
         <v>7</v>
       </c>
-      <c r="N9" s="111"/>
-      <c r="O9" s="112"/>
-      <c r="P9" s="107"/>
-      <c r="Q9" s="106"/>
+      <c r="N9" s="169"/>
+      <c r="O9" s="204"/>
+      <c r="P9" s="167"/>
+      <c r="Q9" s="156"/>
       <c r="R9" s="11"/>
       <c r="S9" s="12"/>
     </row>
     <row r="10" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="103" t="s">
+      <c r="A10" s="155" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="106"/>
-      <c r="C10" s="106"/>
-      <c r="D10" s="106"/>
-      <c r="E10" s="106"/>
-      <c r="F10" s="106"/>
-      <c r="G10" s="104"/>
-      <c r="H10" s="107" t="s">
+      <c r="B10" s="156"/>
+      <c r="C10" s="156"/>
+      <c r="D10" s="156"/>
+      <c r="E10" s="156"/>
+      <c r="F10" s="156"/>
+      <c r="G10" s="165"/>
+      <c r="H10" s="167" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="106"/>
-      <c r="J10" s="106" t="s">
+      <c r="I10" s="156"/>
+      <c r="J10" s="156" t="s">
         <v>10</v>
       </c>
-      <c r="K10" s="106"/>
-      <c r="L10" s="106"/>
+      <c r="K10" s="156"/>
+      <c r="L10" s="156"/>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
       <c r="O10" s="9"/>
@@ -2259,67 +2259,67 @@
       <c r="S10" s="14"/>
     </row>
     <row r="11" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="103" t="s">
+      <c r="A11" s="155" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="106"/>
-      <c r="C11" s="108"/>
-      <c r="D11" s="108"/>
-      <c r="E11" s="108"/>
-      <c r="F11" s="109"/>
-      <c r="G11" s="107" t="s">
+      <c r="B11" s="156"/>
+      <c r="C11" s="158"/>
+      <c r="D11" s="158"/>
+      <c r="E11" s="158"/>
+      <c r="F11" s="166"/>
+      <c r="G11" s="167" t="s">
         <v>12</v>
       </c>
-      <c r="H11" s="106"/>
-      <c r="I11" s="108"/>
-      <c r="J11" s="108"/>
-      <c r="K11" s="108"/>
-      <c r="L11" s="109"/>
-      <c r="M11" s="113" t="s">
+      <c r="H11" s="156"/>
+      <c r="I11" s="158"/>
+      <c r="J11" s="158"/>
+      <c r="K11" s="158"/>
+      <c r="L11" s="166"/>
+      <c r="M11" s="171" t="s">
         <v>13</v>
       </c>
-      <c r="N11" s="114"/>
-      <c r="O11" s="106" t="s">
+      <c r="N11" s="172"/>
+      <c r="O11" s="156" t="s">
         <v>14</v>
       </c>
-      <c r="P11" s="106"/>
-      <c r="Q11" s="106"/>
-      <c r="R11" s="106"/>
-      <c r="S11" s="115"/>
+      <c r="P11" s="156"/>
+      <c r="Q11" s="156"/>
+      <c r="R11" s="156"/>
+      <c r="S11" s="163"/>
     </row>
     <row r="12" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="103" t="s">
+      <c r="A12" s="155" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="106"/>
-      <c r="C12" s="106"/>
-      <c r="D12" s="116"/>
-      <c r="E12" s="106"/>
-      <c r="F12" s="106"/>
-      <c r="G12" s="106"/>
-      <c r="H12" s="106"/>
-      <c r="I12" s="106"/>
-      <c r="J12" s="106"/>
-      <c r="K12" s="106"/>
-      <c r="L12" s="106"/>
-      <c r="M12" s="106"/>
-      <c r="N12" s="106"/>
-      <c r="O12" s="106"/>
-      <c r="P12" s="106"/>
-      <c r="Q12" s="106"/>
-      <c r="R12" s="106"/>
-      <c r="S12" s="115"/>
+      <c r="B12" s="156"/>
+      <c r="C12" s="156"/>
+      <c r="D12" s="164"/>
+      <c r="E12" s="156"/>
+      <c r="F12" s="156"/>
+      <c r="G12" s="156"/>
+      <c r="H12" s="156"/>
+      <c r="I12" s="156"/>
+      <c r="J12" s="156"/>
+      <c r="K12" s="156"/>
+      <c r="L12" s="156"/>
+      <c r="M12" s="156"/>
+      <c r="N12" s="156"/>
+      <c r="O12" s="156"/>
+      <c r="P12" s="156"/>
+      <c r="Q12" s="156"/>
+      <c r="R12" s="156"/>
+      <c r="S12" s="163"/>
     </row>
     <row r="13" spans="1:21" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="106"/>
-      <c r="C13" s="106"/>
-      <c r="D13" s="106"/>
-      <c r="E13" s="106"/>
-      <c r="F13" s="106"/>
-      <c r="G13" s="104"/>
+      <c r="B13" s="156"/>
+      <c r="C13" s="156"/>
+      <c r="D13" s="156"/>
+      <c r="E13" s="156"/>
+      <c r="F13" s="156"/>
+      <c r="G13" s="165"/>
       <c r="H13" s="16" t="s">
         <v>17</v>
       </c>
@@ -2331,89 +2331,89 @@
       <c r="N13" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="O13" s="108"/>
-      <c r="P13" s="108"/>
-      <c r="Q13" s="109"/>
+      <c r="O13" s="158"/>
+      <c r="P13" s="158"/>
+      <c r="Q13" s="166"/>
       <c r="R13" s="18" t="s">
         <v>19</v>
       </c>
       <c r="S13" s="14"/>
     </row>
     <row r="14" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="103" t="s">
+      <c r="A14" s="155" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="106"/>
-      <c r="C14" s="106"/>
-      <c r="D14" s="108"/>
-      <c r="E14" s="108"/>
-      <c r="F14" s="109"/>
-      <c r="G14" s="107" t="s">
+      <c r="B14" s="156"/>
+      <c r="C14" s="156"/>
+      <c r="D14" s="158"/>
+      <c r="E14" s="158"/>
+      <c r="F14" s="166"/>
+      <c r="G14" s="167" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="106"/>
-      <c r="I14" s="106"/>
-      <c r="J14" s="106"/>
-      <c r="K14" s="106" t="s">
+      <c r="H14" s="156"/>
+      <c r="I14" s="156"/>
+      <c r="J14" s="156"/>
+      <c r="K14" s="156" t="s">
         <v>14</v>
       </c>
-      <c r="L14" s="106"/>
-      <c r="M14" s="104"/>
-      <c r="N14" s="110" t="s">
+      <c r="L14" s="156"/>
+      <c r="M14" s="165"/>
+      <c r="N14" s="168" t="s">
         <v>22</v>
       </c>
-      <c r="O14" s="111"/>
-      <c r="P14" s="111"/>
-      <c r="Q14" s="111" t="s">
+      <c r="O14" s="169"/>
+      <c r="P14" s="169"/>
+      <c r="Q14" s="169" t="s">
         <v>14</v>
       </c>
-      <c r="R14" s="111"/>
-      <c r="S14" s="117"/>
+      <c r="R14" s="169"/>
+      <c r="S14" s="170"/>
     </row>
     <row r="15" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="103" t="s">
+      <c r="A15" s="155" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="106"/>
-      <c r="C15" s="106"/>
+      <c r="B15" s="156"/>
+      <c r="C15" s="156"/>
       <c r="D15" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="106" t="s">
+      <c r="E15" s="156" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="106"/>
+      <c r="F15" s="156"/>
       <c r="G15" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="H15" s="106" t="s">
+      <c r="H15" s="156" t="s">
         <v>27</v>
       </c>
-      <c r="I15" s="106"/>
+      <c r="I15" s="156"/>
       <c r="J15" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="K15" s="118" t="s">
+      <c r="K15" s="157" t="s">
         <v>29</v>
       </c>
-      <c r="L15" s="118"/>
+      <c r="L15" s="157"/>
       <c r="M15" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="N15" s="108" t="s">
+      <c r="N15" s="158" t="s">
         <v>31</v>
       </c>
-      <c r="O15" s="108"/>
-      <c r="P15" s="108"/>
-      <c r="Q15" s="119"/>
-      <c r="R15" s="119"/>
-      <c r="S15" s="120"/>
+      <c r="O15" s="158"/>
+      <c r="P15" s="158"/>
+      <c r="Q15" s="159"/>
+      <c r="R15" s="159"/>
+      <c r="S15" s="160"/>
     </row>
     <row r="16" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="103" t="s">
+      <c r="A16" s="155" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="106"/>
+      <c r="B16" s="156"/>
       <c r="C16" s="19" t="s">
         <v>33</v>
       </c>
@@ -2448,19 +2448,19 @@
       <c r="N16" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="O16" s="108" t="s">
+      <c r="O16" s="158" t="s">
         <v>31</v>
       </c>
-      <c r="P16" s="108"/>
-      <c r="Q16" s="108"/>
+      <c r="P16" s="158"/>
+      <c r="Q16" s="158"/>
       <c r="R16" s="13"/>
       <c r="S16" s="20"/>
     </row>
     <row r="17" spans="1:19" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="121" t="s">
+      <c r="A17" s="161" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="122"/>
+      <c r="B17" s="162"/>
       <c r="C17" s="19" t="s">
         <v>35</v>
       </c>
@@ -2478,10 +2478,10 @@
       <c r="I17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J17" s="118" t="s">
+      <c r="J17" s="157" t="s">
         <v>43</v>
       </c>
-      <c r="K17" s="118"/>
+      <c r="K17" s="157"/>
       <c r="L17" s="4"/>
       <c r="M17" s="1" t="s">
         <v>44</v>
@@ -2493,11 +2493,11 @@
       <c r="P17" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="Q17" s="106" t="s">
+      <c r="Q17" s="156" t="s">
         <v>31</v>
       </c>
-      <c r="R17" s="106"/>
-      <c r="S17" s="115"/>
+      <c r="R17" s="156"/>
+      <c r="S17" s="163"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="22"/>
@@ -2518,73 +2518,73 @@
       <c r="S18" s="31"/>
     </row>
     <row r="19" spans="1:19" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="123" t="s">
+      <c r="A19" s="88" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
-      <c r="F19" s="124"/>
-      <c r="G19" s="124"/>
-      <c r="H19" s="124"/>
-      <c r="I19" s="124"/>
-      <c r="J19" s="124"/>
-      <c r="K19" s="124"/>
-      <c r="L19" s="124"/>
-      <c r="M19" s="124"/>
-      <c r="N19" s="124"/>
-      <c r="O19" s="124"/>
-      <c r="P19" s="124"/>
-      <c r="Q19" s="124"/>
-      <c r="R19" s="124"/>
-      <c r="S19" s="125"/>
+      <c r="B19" s="89"/>
+      <c r="C19" s="89"/>
+      <c r="D19" s="89"/>
+      <c r="E19" s="89"/>
+      <c r="F19" s="89"/>
+      <c r="G19" s="89"/>
+      <c r="H19" s="89"/>
+      <c r="I19" s="89"/>
+      <c r="J19" s="89"/>
+      <c r="K19" s="89"/>
+      <c r="L19" s="89"/>
+      <c r="M19" s="89"/>
+      <c r="N19" s="89"/>
+      <c r="O19" s="89"/>
+      <c r="P19" s="89"/>
+      <c r="Q19" s="89"/>
+      <c r="R19" s="89"/>
+      <c r="S19" s="90"/>
     </row>
     <row r="20" spans="1:19" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="126" t="s">
+      <c r="A20" s="138" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="127"/>
-      <c r="C20" s="127"/>
-      <c r="D20" s="127"/>
-      <c r="E20" s="127"/>
-      <c r="F20" s="127"/>
-      <c r="G20" s="127"/>
-      <c r="H20" s="127"/>
-      <c r="I20" s="127"/>
-      <c r="J20" s="127"/>
-      <c r="K20" s="127"/>
-      <c r="L20" s="127"/>
-      <c r="M20" s="127"/>
-      <c r="N20" s="127"/>
-      <c r="O20" s="127"/>
-      <c r="P20" s="127"/>
-      <c r="Q20" s="127"/>
-      <c r="R20" s="127"/>
-      <c r="S20" s="128"/>
+      <c r="B20" s="139"/>
+      <c r="C20" s="139"/>
+      <c r="D20" s="139"/>
+      <c r="E20" s="139"/>
+      <c r="F20" s="139"/>
+      <c r="G20" s="139"/>
+      <c r="H20" s="139"/>
+      <c r="I20" s="139"/>
+      <c r="J20" s="139"/>
+      <c r="K20" s="139"/>
+      <c r="L20" s="139"/>
+      <c r="M20" s="139"/>
+      <c r="N20" s="139"/>
+      <c r="O20" s="139"/>
+      <c r="P20" s="139"/>
+      <c r="Q20" s="139"/>
+      <c r="R20" s="139"/>
+      <c r="S20" s="140"/>
     </row>
     <row r="21" spans="1:19" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="129" t="s">
+      <c r="A21" s="121" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="130"/>
-      <c r="C21" s="130"/>
-      <c r="D21" s="130"/>
-      <c r="E21" s="130"/>
-      <c r="F21" s="130"/>
-      <c r="G21" s="130"/>
-      <c r="H21" s="130"/>
-      <c r="I21" s="130"/>
-      <c r="J21" s="130"/>
-      <c r="K21" s="130"/>
-      <c r="L21" s="130"/>
-      <c r="M21" s="130"/>
-      <c r="N21" s="130"/>
-      <c r="O21" s="130"/>
-      <c r="P21" s="130"/>
-      <c r="Q21" s="130"/>
-      <c r="R21" s="130"/>
-      <c r="S21" s="131"/>
+      <c r="B21" s="122"/>
+      <c r="C21" s="122"/>
+      <c r="D21" s="122"/>
+      <c r="E21" s="122"/>
+      <c r="F21" s="122"/>
+      <c r="G21" s="122"/>
+      <c r="H21" s="122"/>
+      <c r="I21" s="122"/>
+      <c r="J21" s="122"/>
+      <c r="K21" s="122"/>
+      <c r="L21" s="122"/>
+      <c r="M21" s="122"/>
+      <c r="N21" s="122"/>
+      <c r="O21" s="122"/>
+      <c r="P21" s="122"/>
+      <c r="Q21" s="122"/>
+      <c r="R21" s="122"/>
+      <c r="S21" s="123"/>
     </row>
     <row r="22" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
@@ -2599,10 +2599,10 @@
       <c r="D22" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="132" t="s">
+      <c r="E22" s="141" t="s">
         <v>54</v>
       </c>
-      <c r="F22" s="133"/>
+      <c r="F22" s="142"/>
       <c r="G22" s="33" t="s">
         <v>55</v>
       </c>
@@ -2636,10 +2636,10 @@
       <c r="Q22" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="R22" s="132" t="s">
+      <c r="R22" s="141" t="s">
         <v>66</v>
       </c>
-      <c r="S22" s="134"/>
+      <c r="S22" s="143"/>
     </row>
     <row r="23" spans="1:19" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="34"/>
@@ -2873,23 +2873,23 @@
       <c r="S33" s="41"/>
     </row>
     <row r="34" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A34" s="135" t="s">
+      <c r="A34" s="144" t="s">
         <v>67</v>
       </c>
-      <c r="B34" s="136"/>
-      <c r="C34" s="136"/>
-      <c r="D34" s="136"/>
-      <c r="E34" s="136"/>
-      <c r="F34" s="136"/>
-      <c r="G34" s="136"/>
-      <c r="H34" s="136"/>
-      <c r="I34" s="136"/>
-      <c r="J34" s="136"/>
-      <c r="K34" s="136"/>
-      <c r="L34" s="136"/>
-      <c r="M34" s="136"/>
-      <c r="N34" s="136"/>
-      <c r="O34" s="136"/>
+      <c r="B34" s="145"/>
+      <c r="C34" s="145"/>
+      <c r="D34" s="145"/>
+      <c r="E34" s="145"/>
+      <c r="F34" s="145"/>
+      <c r="G34" s="145"/>
+      <c r="H34" s="145"/>
+      <c r="I34" s="145"/>
+      <c r="J34" s="145"/>
+      <c r="K34" s="145"/>
+      <c r="L34" s="145"/>
+      <c r="M34" s="145"/>
+      <c r="N34" s="145"/>
+      <c r="O34" s="145"/>
       <c r="P34" s="45"/>
       <c r="Q34" s="45"/>
       <c r="R34" s="45"/>
@@ -2897,21 +2897,21 @@
       <c r="T34" s="47"/>
     </row>
     <row r="35" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="137"/>
-      <c r="B35" s="138"/>
-      <c r="C35" s="138"/>
-      <c r="D35" s="138"/>
-      <c r="E35" s="138"/>
-      <c r="F35" s="138"/>
-      <c r="G35" s="138"/>
-      <c r="H35" s="138"/>
-      <c r="I35" s="138"/>
-      <c r="J35" s="138"/>
-      <c r="K35" s="138"/>
-      <c r="L35" s="138"/>
-      <c r="M35" s="138"/>
-      <c r="N35" s="138"/>
-      <c r="O35" s="138"/>
+      <c r="A35" s="146"/>
+      <c r="B35" s="147"/>
+      <c r="C35" s="147"/>
+      <c r="D35" s="147"/>
+      <c r="E35" s="147"/>
+      <c r="F35" s="147"/>
+      <c r="G35" s="147"/>
+      <c r="H35" s="147"/>
+      <c r="I35" s="147"/>
+      <c r="J35" s="147"/>
+      <c r="K35" s="147"/>
+      <c r="L35" s="147"/>
+      <c r="M35" s="147"/>
+      <c r="N35" s="147"/>
+      <c r="O35" s="147"/>
       <c r="S35" s="48"/>
       <c r="T35" s="47"/>
     </row>
@@ -2922,18 +2922,18 @@
       <c r="D36" s="50"/>
       <c r="E36" s="50"/>
       <c r="F36" s="50"/>
-      <c r="G36" s="139" t="s">
+      <c r="G36" s="148" t="s">
         <v>68</v>
       </c>
-      <c r="H36" s="140"/>
-      <c r="I36" s="140"/>
-      <c r="J36" s="141"/>
-      <c r="K36" s="139" t="s">
+      <c r="H36" s="149"/>
+      <c r="I36" s="149"/>
+      <c r="J36" s="150"/>
+      <c r="K36" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="L36" s="140"/>
-      <c r="M36" s="140"/>
-      <c r="N36" s="141"/>
+      <c r="L36" s="149"/>
+      <c r="M36" s="149"/>
+      <c r="N36" s="150"/>
       <c r="O36" s="47"/>
       <c r="P36" s="47"/>
       <c r="Q36" s="47"/>
@@ -2942,28 +2942,22 @@
       <c r="T36" s="47"/>
     </row>
     <row r="37" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A37" s="142" t="s">
+      <c r="A37" s="151" t="s">
         <v>70</v>
       </c>
-      <c r="B37" s="143"/>
-      <c r="C37" s="143"/>
-      <c r="D37" s="143"/>
-      <c r="E37" s="143"/>
-      <c r="F37" s="144"/>
-      <c r="G37" s="145">
-        <f>SUM(O23:O29,O31:O33)</f>
-        <v>0</v>
-      </c>
-      <c r="H37" s="146"/>
-      <c r="I37" s="146"/>
-      <c r="J37" s="147"/>
-      <c r="K37" s="148">
-        <f>SUM(Q23:Q28)</f>
-        <v>0</v>
-      </c>
-      <c r="L37" s="149"/>
-      <c r="M37" s="149"/>
-      <c r="N37" s="150"/>
+      <c r="B37" s="112"/>
+      <c r="C37" s="112"/>
+      <c r="D37" s="112"/>
+      <c r="E37" s="112"/>
+      <c r="F37" s="113"/>
+      <c r="G37" s="118"/>
+      <c r="H37" s="119"/>
+      <c r="I37" s="119"/>
+      <c r="J37" s="120"/>
+      <c r="K37" s="152"/>
+      <c r="L37" s="153"/>
+      <c r="M37" s="153"/>
+      <c r="N37" s="154"/>
       <c r="O37" s="47"/>
       <c r="P37" s="47"/>
       <c r="Q37" s="47"/>
@@ -2971,28 +2965,22 @@
       <c r="S37" s="51"/>
     </row>
     <row r="38" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A38" s="151" t="s">
+      <c r="A38" s="111" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="143"/>
-      <c r="C38" s="143"/>
-      <c r="D38" s="143"/>
-      <c r="E38" s="143"/>
-      <c r="F38" s="144"/>
-      <c r="G38" s="145">
-        <f>4-G37</f>
-        <v>4</v>
-      </c>
-      <c r="H38" s="146"/>
-      <c r="I38" s="146"/>
-      <c r="J38" s="147"/>
-      <c r="K38" s="145">
-        <f>4-K37</f>
-        <v>4</v>
-      </c>
-      <c r="L38" s="146"/>
-      <c r="M38" s="146"/>
-      <c r="N38" s="147"/>
+      <c r="B38" s="112"/>
+      <c r="C38" s="112"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="113"/>
+      <c r="G38" s="118"/>
+      <c r="H38" s="119"/>
+      <c r="I38" s="119"/>
+      <c r="J38" s="120"/>
+      <c r="K38" s="118"/>
+      <c r="L38" s="119"/>
+      <c r="M38" s="119"/>
+      <c r="N38" s="120"/>
       <c r="O38" s="47"/>
       <c r="P38" s="47"/>
       <c r="Q38" s="47"/>
@@ -3000,28 +2988,22 @@
       <c r="S38" s="51"/>
     </row>
     <row r="39" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A39" s="152" t="s">
+      <c r="A39" s="132" t="s">
         <v>72</v>
       </c>
-      <c r="B39" s="153"/>
-      <c r="C39" s="153"/>
-      <c r="D39" s="153"/>
-      <c r="E39" s="153"/>
-      <c r="F39" s="154"/>
-      <c r="G39" s="145">
-        <f>G37</f>
-        <v>0</v>
-      </c>
-      <c r="H39" s="146"/>
-      <c r="I39" s="146"/>
-      <c r="J39" s="147"/>
-      <c r="K39" s="145">
-        <f>K37</f>
-        <v>0</v>
-      </c>
-      <c r="L39" s="146"/>
-      <c r="M39" s="146"/>
-      <c r="N39" s="147"/>
+      <c r="B39" s="133"/>
+      <c r="C39" s="133"/>
+      <c r="D39" s="133"/>
+      <c r="E39" s="133"/>
+      <c r="F39" s="134"/>
+      <c r="G39" s="118"/>
+      <c r="H39" s="119"/>
+      <c r="I39" s="119"/>
+      <c r="J39" s="120"/>
+      <c r="K39" s="118"/>
+      <c r="L39" s="119"/>
+      <c r="M39" s="119"/>
+      <c r="N39" s="120"/>
       <c r="O39" s="47"/>
       <c r="P39" s="47"/>
       <c r="Q39" s="47"/>
@@ -3029,26 +3011,26 @@
       <c r="S39" s="51"/>
     </row>
     <row r="40" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="155" t="s">
+      <c r="A40" s="135" t="s">
         <v>73</v>
       </c>
-      <c r="B40" s="156"/>
-      <c r="C40" s="156"/>
-      <c r="D40" s="156"/>
-      <c r="E40" s="156"/>
-      <c r="F40" s="157"/>
-      <c r="G40" s="158" t="s">
+      <c r="B40" s="136"/>
+      <c r="C40" s="136"/>
+      <c r="D40" s="136"/>
+      <c r="E40" s="136"/>
+      <c r="F40" s="137"/>
+      <c r="G40" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="H40" s="159"/>
-      <c r="I40" s="159"/>
-      <c r="J40" s="160"/>
-      <c r="K40" s="158" t="s">
+      <c r="H40" s="98"/>
+      <c r="I40" s="98"/>
+      <c r="J40" s="99"/>
+      <c r="K40" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="L40" s="159"/>
-      <c r="M40" s="159"/>
-      <c r="N40" s="160"/>
+      <c r="L40" s="98"/>
+      <c r="M40" s="98"/>
+      <c r="N40" s="99"/>
       <c r="O40" s="47"/>
       <c r="P40" s="47"/>
       <c r="Q40" s="47"/>
@@ -3056,26 +3038,26 @@
       <c r="S40" s="51"/>
     </row>
     <row r="41" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41" s="151" t="s">
+      <c r="A41" s="111" t="s">
         <v>74</v>
       </c>
-      <c r="B41" s="143"/>
-      <c r="C41" s="143"/>
-      <c r="D41" s="143"/>
-      <c r="E41" s="143"/>
-      <c r="F41" s="144"/>
-      <c r="G41" s="158" t="s">
+      <c r="B41" s="112"/>
+      <c r="C41" s="112"/>
+      <c r="D41" s="112"/>
+      <c r="E41" s="112"/>
+      <c r="F41" s="113"/>
+      <c r="G41" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="H41" s="159"/>
-      <c r="I41" s="159"/>
-      <c r="J41" s="160"/>
-      <c r="K41" s="158" t="s">
+      <c r="H41" s="98"/>
+      <c r="I41" s="98"/>
+      <c r="J41" s="99"/>
+      <c r="K41" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="L41" s="159"/>
-      <c r="M41" s="159"/>
-      <c r="N41" s="160"/>
+      <c r="L41" s="98"/>
+      <c r="M41" s="98"/>
+      <c r="N41" s="99"/>
       <c r="O41" s="47"/>
       <c r="P41" s="47"/>
       <c r="Q41" s="47"/>
@@ -3083,28 +3065,28 @@
       <c r="S41" s="51"/>
     </row>
     <row r="42" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A42" s="161" t="s">
+      <c r="A42" s="115" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="162"/>
-      <c r="C42" s="162"/>
-      <c r="D42" s="162"/>
-      <c r="E42" s="162"/>
-      <c r="F42" s="163"/>
-      <c r="G42" s="145">
+      <c r="B42" s="116"/>
+      <c r="C42" s="116"/>
+      <c r="D42" s="116"/>
+      <c r="E42" s="116"/>
+      <c r="F42" s="117"/>
+      <c r="G42" s="118">
         <f>G37</f>
         <v>0</v>
       </c>
-      <c r="H42" s="146"/>
-      <c r="I42" s="146"/>
-      <c r="J42" s="147"/>
-      <c r="K42" s="145">
+      <c r="H42" s="119"/>
+      <c r="I42" s="119"/>
+      <c r="J42" s="120"/>
+      <c r="K42" s="118">
         <f>K37</f>
         <v>0</v>
       </c>
-      <c r="L42" s="159"/>
-      <c r="M42" s="159"/>
-      <c r="N42" s="160"/>
+      <c r="L42" s="98"/>
+      <c r="M42" s="98"/>
+      <c r="N42" s="99"/>
       <c r="O42" s="47"/>
       <c r="P42" s="47"/>
       <c r="Q42" s="47"/>
@@ -3133,144 +3115,144 @@
       <c r="S43" s="54"/>
     </row>
     <row r="44" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A44" s="129" t="s">
+      <c r="A44" s="121" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="130"/>
-      <c r="C44" s="130"/>
-      <c r="D44" s="130"/>
-      <c r="E44" s="130"/>
-      <c r="F44" s="130"/>
-      <c r="G44" s="130"/>
-      <c r="H44" s="130"/>
-      <c r="I44" s="130"/>
-      <c r="J44" s="130"/>
-      <c r="K44" s="130"/>
-      <c r="L44" s="130"/>
-      <c r="M44" s="130"/>
-      <c r="N44" s="130"/>
-      <c r="O44" s="130"/>
-      <c r="P44" s="130"/>
-      <c r="Q44" s="130"/>
-      <c r="R44" s="130"/>
-      <c r="S44" s="131"/>
+      <c r="B44" s="122"/>
+      <c r="C44" s="122"/>
+      <c r="D44" s="122"/>
+      <c r="E44" s="122"/>
+      <c r="F44" s="122"/>
+      <c r="G44" s="122"/>
+      <c r="H44" s="122"/>
+      <c r="I44" s="122"/>
+      <c r="J44" s="122"/>
+      <c r="K44" s="122"/>
+      <c r="L44" s="122"/>
+      <c r="M44" s="122"/>
+      <c r="N44" s="122"/>
+      <c r="O44" s="122"/>
+      <c r="P44" s="122"/>
+      <c r="Q44" s="122"/>
+      <c r="R44" s="122"/>
+      <c r="S44" s="123"/>
     </row>
     <row r="45" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="164" t="s">
+      <c r="A45" s="124" t="s">
         <v>51</v>
       </c>
-      <c r="B45" s="165"/>
-      <c r="C45" s="166"/>
-      <c r="D45" s="167" t="s">
+      <c r="B45" s="125"/>
+      <c r="C45" s="126"/>
+      <c r="D45" s="127" t="s">
         <v>53</v>
       </c>
-      <c r="E45" s="168"/>
-      <c r="F45" s="169"/>
-      <c r="G45" s="167" t="s">
+      <c r="E45" s="128"/>
+      <c r="F45" s="129"/>
+      <c r="G45" s="127" t="s">
         <v>54</v>
       </c>
-      <c r="H45" s="168"/>
-      <c r="I45" s="169"/>
+      <c r="H45" s="128"/>
+      <c r="I45" s="129"/>
       <c r="J45" s="55" t="s">
         <v>55</v>
       </c>
-      <c r="K45" s="170" t="s">
+      <c r="K45" s="130" t="s">
         <v>77</v>
       </c>
-      <c r="L45" s="165"/>
-      <c r="M45" s="166"/>
-      <c r="N45" s="170" t="s">
+      <c r="L45" s="125"/>
+      <c r="M45" s="126"/>
+      <c r="N45" s="130" t="s">
         <v>78</v>
       </c>
-      <c r="O45" s="166"/>
-      <c r="P45" s="167" t="s">
+      <c r="O45" s="126"/>
+      <c r="P45" s="127" t="s">
         <v>66</v>
       </c>
-      <c r="Q45" s="168"/>
-      <c r="R45" s="168"/>
-      <c r="S45" s="171"/>
+      <c r="Q45" s="128"/>
+      <c r="R45" s="128"/>
+      <c r="S45" s="131"/>
     </row>
     <row r="46" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A46" s="172" t="s">
+      <c r="A46" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="B46" s="173"/>
-      <c r="C46" s="174"/>
-      <c r="D46" s="175" t="s">
+      <c r="B46" s="107"/>
+      <c r="C46" s="108"/>
+      <c r="D46" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="E46" s="173"/>
-      <c r="F46" s="174"/>
-      <c r="G46" s="175" t="s">
+      <c r="E46" s="107"/>
+      <c r="F46" s="108"/>
+      <c r="G46" s="109" t="s">
         <v>80</v>
       </c>
-      <c r="H46" s="173"/>
-      <c r="I46" s="174"/>
+      <c r="H46" s="107"/>
+      <c r="I46" s="108"/>
       <c r="J46" s="56">
         <v>1</v>
       </c>
-      <c r="K46" s="175"/>
-      <c r="L46" s="173"/>
-      <c r="M46" s="174"/>
-      <c r="N46" s="175" t="s">
+      <c r="K46" s="109"/>
+      <c r="L46" s="107"/>
+      <c r="M46" s="108"/>
+      <c r="N46" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="O46" s="174"/>
-      <c r="P46" s="175" t="s">
+      <c r="O46" s="108"/>
+      <c r="P46" s="109" t="s">
         <v>80</v>
       </c>
-      <c r="Q46" s="173"/>
-      <c r="R46" s="173"/>
-      <c r="S46" s="176"/>
+      <c r="Q46" s="107"/>
+      <c r="R46" s="107"/>
+      <c r="S46" s="110"/>
     </row>
     <row r="47" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A47" s="172" t="s">
+      <c r="A47" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="B47" s="173"/>
-      <c r="C47" s="174"/>
-      <c r="D47" s="175" t="s">
+      <c r="B47" s="107"/>
+      <c r="C47" s="108"/>
+      <c r="D47" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="E47" s="173"/>
-      <c r="F47" s="174"/>
-      <c r="G47" s="175" t="s">
+      <c r="E47" s="107"/>
+      <c r="F47" s="108"/>
+      <c r="G47" s="109" t="s">
         <v>81</v>
       </c>
-      <c r="H47" s="173"/>
-      <c r="I47" s="174"/>
+      <c r="H47" s="107"/>
+      <c r="I47" s="108"/>
       <c r="J47" s="56">
         <v>1</v>
       </c>
-      <c r="K47" s="175" t="s">
+      <c r="K47" s="109" t="s">
         <v>82</v>
       </c>
-      <c r="L47" s="173"/>
-      <c r="M47" s="174"/>
-      <c r="N47" s="175" t="s">
+      <c r="L47" s="107"/>
+      <c r="M47" s="108"/>
+      <c r="N47" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="O47" s="174"/>
-      <c r="P47" s="175" t="s">
+      <c r="O47" s="108"/>
+      <c r="P47" s="109" t="s">
         <v>81</v>
       </c>
-      <c r="Q47" s="173"/>
-      <c r="R47" s="173"/>
-      <c r="S47" s="176"/>
+      <c r="Q47" s="107"/>
+      <c r="R47" s="107"/>
+      <c r="S47" s="110"/>
     </row>
     <row r="48" spans="1:20" ht="15" x14ac:dyDescent="0.25">
-      <c r="A48" s="177" t="s">
+      <c r="A48" s="97" t="s">
         <v>83</v>
       </c>
-      <c r="B48" s="159"/>
-      <c r="C48" s="159"/>
-      <c r="D48" s="159"/>
-      <c r="E48" s="159"/>
-      <c r="F48" s="159"/>
-      <c r="G48" s="159"/>
-      <c r="H48" s="159"/>
-      <c r="I48" s="159"/>
-      <c r="J48" s="160"/>
+      <c r="B48" s="98"/>
+      <c r="C48" s="98"/>
+      <c r="D48" s="98"/>
+      <c r="E48" s="98"/>
+      <c r="F48" s="98"/>
+      <c r="G48" s="98"/>
+      <c r="H48" s="98"/>
+      <c r="I48" s="98"/>
+      <c r="J48" s="99"/>
       <c r="K48" s="47"/>
       <c r="L48" s="47"/>
       <c r="M48" s="47"/>
@@ -3282,106 +3264,106 @@
       <c r="S48" s="52"/>
     </row>
     <row r="49" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="178" t="s">
+      <c r="A49" s="79" t="s">
         <v>84</v>
       </c>
-      <c r="B49" s="179"/>
-      <c r="C49" s="179"/>
-      <c r="D49" s="180"/>
-      <c r="E49" s="181"/>
-      <c r="F49" s="182"/>
-      <c r="G49" s="182"/>
-      <c r="H49" s="182"/>
-      <c r="I49" s="182"/>
-      <c r="J49" s="183"/>
+      <c r="B49" s="80"/>
+      <c r="C49" s="80"/>
+      <c r="D49" s="81"/>
+      <c r="E49" s="82"/>
+      <c r="F49" s="83"/>
+      <c r="G49" s="83"/>
+      <c r="H49" s="83"/>
+      <c r="I49" s="83"/>
+      <c r="J49" s="84"/>
       <c r="S49" s="57"/>
     </row>
     <row r="50" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="178" t="s">
+      <c r="A50" s="79" t="s">
         <v>85</v>
       </c>
-      <c r="B50" s="179"/>
-      <c r="C50" s="179"/>
-      <c r="D50" s="180"/>
-      <c r="E50" s="181">
+      <c r="B50" s="80"/>
+      <c r="C50" s="80"/>
+      <c r="D50" s="81"/>
+      <c r="E50" s="82">
         <f>10-E49</f>
         <v>10</v>
       </c>
-      <c r="F50" s="182"/>
-      <c r="G50" s="182"/>
-      <c r="H50" s="182"/>
-      <c r="I50" s="182"/>
-      <c r="J50" s="183"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="83"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="83"/>
+      <c r="J50" s="84"/>
       <c r="S50" s="57"/>
     </row>
     <row r="51" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A51" s="184" t="s">
+      <c r="A51" s="100" t="s">
         <v>86</v>
       </c>
-      <c r="B51" s="185"/>
-      <c r="C51" s="185"/>
-      <c r="D51" s="186"/>
-      <c r="E51" s="181">
+      <c r="B51" s="101"/>
+      <c r="C51" s="101"/>
+      <c r="D51" s="102"/>
+      <c r="E51" s="82">
         <f>E49</f>
         <v>0</v>
       </c>
-      <c r="F51" s="182"/>
-      <c r="G51" s="182"/>
-      <c r="H51" s="182"/>
-      <c r="I51" s="182"/>
-      <c r="J51" s="183"/>
+      <c r="F51" s="83"/>
+      <c r="G51" s="83"/>
+      <c r="H51" s="83"/>
+      <c r="I51" s="83"/>
+      <c r="J51" s="84"/>
       <c r="S51" s="57"/>
     </row>
     <row r="52" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52" s="187" t="s">
+      <c r="A52" s="103" t="s">
         <v>87</v>
       </c>
-      <c r="B52" s="188"/>
-      <c r="C52" s="188"/>
-      <c r="D52" s="189"/>
-      <c r="E52" s="181" t="s">
+      <c r="B52" s="104"/>
+      <c r="C52" s="104"/>
+      <c r="D52" s="105"/>
+      <c r="E52" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="F52" s="182"/>
-      <c r="G52" s="182"/>
-      <c r="H52" s="182"/>
-      <c r="I52" s="182"/>
-      <c r="J52" s="183"/>
+      <c r="F52" s="83"/>
+      <c r="G52" s="83"/>
+      <c r="H52" s="83"/>
+      <c r="I52" s="83"/>
+      <c r="J52" s="84"/>
       <c r="S52" s="57"/>
     </row>
     <row r="53" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53" s="178" t="s">
+      <c r="A53" s="79" t="s">
         <v>88</v>
       </c>
-      <c r="B53" s="179"/>
-      <c r="C53" s="179"/>
-      <c r="D53" s="180"/>
-      <c r="E53" s="181" t="s">
+      <c r="B53" s="80"/>
+      <c r="C53" s="80"/>
+      <c r="D53" s="81"/>
+      <c r="E53" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="F53" s="182"/>
-      <c r="G53" s="182"/>
-      <c r="H53" s="182"/>
-      <c r="I53" s="182"/>
-      <c r="J53" s="183"/>
+      <c r="F53" s="83"/>
+      <c r="G53" s="83"/>
+      <c r="H53" s="83"/>
+      <c r="I53" s="83"/>
+      <c r="J53" s="84"/>
       <c r="S53" s="57"/>
     </row>
     <row r="54" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54" s="190" t="s">
+      <c r="A54" s="85" t="s">
         <v>89</v>
       </c>
-      <c r="B54" s="191"/>
-      <c r="C54" s="191"/>
-      <c r="D54" s="192"/>
-      <c r="E54" s="181">
+      <c r="B54" s="86"/>
+      <c r="C54" s="86"/>
+      <c r="D54" s="87"/>
+      <c r="E54" s="82">
         <f>E49</f>
         <v>0</v>
       </c>
-      <c r="F54" s="182"/>
-      <c r="G54" s="182"/>
-      <c r="H54" s="182"/>
-      <c r="I54" s="182"/>
-      <c r="J54" s="183"/>
+      <c r="F54" s="83"/>
+      <c r="G54" s="83"/>
+      <c r="H54" s="83"/>
+      <c r="I54" s="83"/>
+      <c r="J54" s="84"/>
       <c r="S54" s="57"/>
     </row>
     <row r="55" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3389,54 +3371,54 @@
       <c r="S55" s="57"/>
     </row>
     <row r="56" spans="1:26" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="123" t="s">
+      <c r="A56" s="88" t="s">
         <v>66</v>
       </c>
-      <c r="B56" s="124"/>
-      <c r="C56" s="124"/>
-      <c r="D56" s="124"/>
-      <c r="E56" s="124"/>
-      <c r="F56" s="124"/>
-      <c r="G56" s="124"/>
-      <c r="H56" s="124"/>
-      <c r="I56" s="124"/>
-      <c r="J56" s="124"/>
-      <c r="K56" s="124"/>
-      <c r="L56" s="124"/>
-      <c r="M56" s="124"/>
-      <c r="N56" s="124"/>
-      <c r="O56" s="124"/>
-      <c r="P56" s="124"/>
-      <c r="Q56" s="124"/>
-      <c r="R56" s="124"/>
-      <c r="S56" s="125"/>
+      <c r="B56" s="89"/>
+      <c r="C56" s="89"/>
+      <c r="D56" s="89"/>
+      <c r="E56" s="89"/>
+      <c r="F56" s="89"/>
+      <c r="G56" s="89"/>
+      <c r="H56" s="89"/>
+      <c r="I56" s="89"/>
+      <c r="J56" s="89"/>
+      <c r="K56" s="89"/>
+      <c r="L56" s="89"/>
+      <c r="M56" s="89"/>
+      <c r="N56" s="89"/>
+      <c r="O56" s="89"/>
+      <c r="P56" s="89"/>
+      <c r="Q56" s="89"/>
+      <c r="R56" s="89"/>
+      <c r="S56" s="90"/>
     </row>
     <row r="57" spans="1:26" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="58"/>
       <c r="S57" s="57"/>
     </row>
     <row r="58" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="193" t="s">
+      <c r="A58" s="91" t="s">
         <v>90</v>
       </c>
-      <c r="B58" s="194"/>
-      <c r="C58" s="194"/>
-      <c r="D58" s="194"/>
-      <c r="E58" s="194"/>
-      <c r="F58" s="194"/>
-      <c r="G58" s="194"/>
-      <c r="H58" s="194"/>
-      <c r="I58" s="194"/>
-      <c r="J58" s="194"/>
-      <c r="K58" s="194"/>
-      <c r="L58" s="194"/>
-      <c r="M58" s="194"/>
-      <c r="N58" s="194"/>
-      <c r="O58" s="194"/>
-      <c r="P58" s="194"/>
-      <c r="Q58" s="194"/>
-      <c r="R58" s="194"/>
-      <c r="S58" s="195"/>
+      <c r="B58" s="92"/>
+      <c r="C58" s="92"/>
+      <c r="D58" s="92"/>
+      <c r="E58" s="92"/>
+      <c r="F58" s="92"/>
+      <c r="G58" s="92"/>
+      <c r="H58" s="92"/>
+      <c r="I58" s="92"/>
+      <c r="J58" s="92"/>
+      <c r="K58" s="92"/>
+      <c r="L58" s="92"/>
+      <c r="M58" s="92"/>
+      <c r="N58" s="92"/>
+      <c r="O58" s="92"/>
+      <c r="P58" s="92"/>
+      <c r="Q58" s="92"/>
+      <c r="R58" s="92"/>
+      <c r="S58" s="93"/>
     </row>
     <row r="59" spans="1:26" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="58"/>
@@ -3447,50 +3429,50 @@
       <c r="S60" s="57"/>
     </row>
     <row r="61" spans="1:26" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="123" t="s">
+      <c r="A61" s="88" t="s">
         <v>91</v>
       </c>
-      <c r="B61" s="124"/>
-      <c r="C61" s="124"/>
-      <c r="D61" s="124"/>
-      <c r="E61" s="124"/>
-      <c r="F61" s="124"/>
-      <c r="G61" s="124"/>
-      <c r="H61" s="124"/>
-      <c r="I61" s="124"/>
-      <c r="J61" s="124"/>
-      <c r="K61" s="124"/>
-      <c r="L61" s="124"/>
-      <c r="M61" s="124"/>
-      <c r="N61" s="124"/>
-      <c r="O61" s="124"/>
-      <c r="P61" s="124"/>
-      <c r="Q61" s="124"/>
-      <c r="R61" s="124"/>
-      <c r="S61" s="125"/>
+      <c r="B61" s="89"/>
+      <c r="C61" s="89"/>
+      <c r="D61" s="89"/>
+      <c r="E61" s="89"/>
+      <c r="F61" s="89"/>
+      <c r="G61" s="89"/>
+      <c r="H61" s="89"/>
+      <c r="I61" s="89"/>
+      <c r="J61" s="89"/>
+      <c r="K61" s="89"/>
+      <c r="L61" s="89"/>
+      <c r="M61" s="89"/>
+      <c r="N61" s="89"/>
+      <c r="O61" s="89"/>
+      <c r="P61" s="89"/>
+      <c r="Q61" s="89"/>
+      <c r="R61" s="89"/>
+      <c r="S61" s="90"/>
     </row>
     <row r="62" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A62" s="196" t="s">
+      <c r="A62" s="94" t="s">
         <v>92</v>
       </c>
-      <c r="B62" s="197"/>
-      <c r="C62" s="197"/>
-      <c r="D62" s="197"/>
-      <c r="E62" s="197"/>
-      <c r="F62" s="197"/>
-      <c r="G62" s="197"/>
-      <c r="H62" s="197"/>
-      <c r="I62" s="197"/>
-      <c r="J62" s="197"/>
-      <c r="K62" s="197"/>
-      <c r="L62" s="197"/>
-      <c r="M62" s="197"/>
-      <c r="N62" s="197"/>
-      <c r="O62" s="197"/>
-      <c r="P62" s="197"/>
-      <c r="Q62" s="197"/>
-      <c r="R62" s="197"/>
-      <c r="S62" s="198"/>
+      <c r="B62" s="95"/>
+      <c r="C62" s="95"/>
+      <c r="D62" s="95"/>
+      <c r="E62" s="95"/>
+      <c r="F62" s="95"/>
+      <c r="G62" s="95"/>
+      <c r="H62" s="95"/>
+      <c r="I62" s="95"/>
+      <c r="J62" s="95"/>
+      <c r="K62" s="95"/>
+      <c r="L62" s="95"/>
+      <c r="M62" s="95"/>
+      <c r="N62" s="95"/>
+      <c r="O62" s="95"/>
+      <c r="P62" s="95"/>
+      <c r="Q62" s="95"/>
+      <c r="R62" s="95"/>
+      <c r="S62" s="96"/>
       <c r="W62" s="59"/>
       <c r="X62" s="59"/>
       <c r="Y62" s="59"/>
@@ -3527,12 +3509,12 @@
     </row>
     <row r="65" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="58"/>
-      <c r="J65" s="199" t="s">
+      <c r="J65" s="73" t="s">
         <v>93</v>
       </c>
-      <c r="K65" s="199"/>
-      <c r="L65" s="199"/>
-      <c r="M65" s="199"/>
+      <c r="K65" s="73"/>
+      <c r="L65" s="73"/>
+      <c r="M65" s="73"/>
       <c r="N65" s="64"/>
       <c r="O65" s="64"/>
       <c r="S65" s="57"/>
@@ -3564,11 +3546,11 @@
     <row r="68" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="58"/>
       <c r="H68" s="67"/>
-      <c r="J68" s="199" t="s">
+      <c r="J68" s="73" t="s">
         <v>95</v>
       </c>
-      <c r="K68" s="199"/>
-      <c r="L68" s="199"/>
+      <c r="K68" s="73"/>
+      <c r="L68" s="73"/>
       <c r="M68" s="67"/>
       <c r="N68" s="64"/>
       <c r="O68" s="67"/>
@@ -3597,27 +3579,27 @@
       <c r="S69" s="54"/>
     </row>
     <row r="70" spans="1:19" ht="15" x14ac:dyDescent="0.25">
-      <c r="A70" s="200" t="s">
+      <c r="A70" s="74" t="s">
         <v>96</v>
       </c>
-      <c r="B70" s="201"/>
-      <c r="C70" s="201"/>
-      <c r="D70" s="201"/>
-      <c r="E70" s="201"/>
-      <c r="F70" s="201"/>
-      <c r="G70" s="201"/>
-      <c r="H70" s="201"/>
-      <c r="I70" s="201"/>
-      <c r="J70" s="201"/>
-      <c r="K70" s="201"/>
-      <c r="L70" s="201"/>
-      <c r="M70" s="201"/>
-      <c r="N70" s="201"/>
-      <c r="O70" s="201"/>
-      <c r="P70" s="201"/>
-      <c r="Q70" s="201"/>
-      <c r="R70" s="201"/>
-      <c r="S70" s="202"/>
+      <c r="B70" s="75"/>
+      <c r="C70" s="75"/>
+      <c r="D70" s="75"/>
+      <c r="E70" s="75"/>
+      <c r="F70" s="75"/>
+      <c r="G70" s="75"/>
+      <c r="H70" s="75"/>
+      <c r="I70" s="75"/>
+      <c r="J70" s="75"/>
+      <c r="K70" s="75"/>
+      <c r="L70" s="75"/>
+      <c r="M70" s="75"/>
+      <c r="N70" s="75"/>
+      <c r="O70" s="75"/>
+      <c r="P70" s="75"/>
+      <c r="Q70" s="75"/>
+      <c r="R70" s="75"/>
+      <c r="S70" s="76"/>
     </row>
     <row r="71" spans="1:19" ht="15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="61"/>
@@ -3642,25 +3624,25 @@
     </row>
     <row r="72" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="63"/>
-      <c r="I72" s="203"/>
-      <c r="J72" s="203"/>
-      <c r="K72" s="203"/>
-      <c r="L72" s="203"/>
-      <c r="M72" s="203"/>
+      <c r="I72" s="77"/>
+      <c r="J72" s="77"/>
+      <c r="K72" s="77"/>
+      <c r="L72" s="77"/>
+      <c r="M72" s="77"/>
       <c r="S72" s="57"/>
     </row>
     <row r="73" spans="1:19" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="58"/>
-      <c r="D73" s="199"/>
-      <c r="E73" s="199"/>
-      <c r="F73" s="199"/>
-      <c r="G73" s="199"/>
-      <c r="J73" s="199" t="s">
+      <c r="D73" s="73"/>
+      <c r="E73" s="73"/>
+      <c r="F73" s="73"/>
+      <c r="G73" s="73"/>
+      <c r="J73" s="73" t="s">
         <v>93</v>
       </c>
-      <c r="K73" s="199"/>
-      <c r="L73" s="199"/>
-      <c r="M73" s="199"/>
+      <c r="K73" s="73"/>
+      <c r="L73" s="73"/>
+      <c r="M73" s="73"/>
       <c r="S73" s="57"/>
     </row>
     <row r="74" spans="1:19" ht="15" x14ac:dyDescent="0.25">
@@ -3673,9 +3655,9 @@
         <v>97</v>
       </c>
       <c r="L74" s="65"/>
-      <c r="M74" s="204"/>
-      <c r="N74" s="204"/>
-      <c r="O74" s="204"/>
+      <c r="M74" s="78"/>
+      <c r="N74" s="78"/>
+      <c r="O74" s="78"/>
       <c r="S74" s="57"/>
     </row>
     <row r="75" spans="1:19" ht="15" x14ac:dyDescent="0.25">
@@ -3688,27 +3670,27 @@
         <v>94</v>
       </c>
       <c r="L75" s="65"/>
-      <c r="M75" s="204"/>
-      <c r="N75" s="204"/>
-      <c r="O75" s="204"/>
+      <c r="M75" s="78"/>
+      <c r="N75" s="78"/>
+      <c r="O75" s="78"/>
       <c r="S75" s="57"/>
     </row>
     <row r="76" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A76" s="58"/>
-      <c r="D76" s="199"/>
-      <c r="E76" s="199"/>
-      <c r="F76" s="199"/>
+      <c r="D76" s="73"/>
+      <c r="E76" s="73"/>
+      <c r="F76" s="73"/>
       <c r="G76" s="67"/>
       <c r="H76" s="67"/>
-      <c r="J76" s="199" t="s">
+      <c r="J76" s="73" t="s">
         <v>95</v>
       </c>
-      <c r="K76" s="199"/>
-      <c r="L76" s="199"/>
+      <c r="K76" s="73"/>
+      <c r="L76" s="73"/>
       <c r="M76" s="65"/>
       <c r="N76" s="65"/>
-      <c r="O76" s="204"/>
-      <c r="P76" s="204"/>
+      <c r="O76" s="78"/>
+      <c r="P76" s="78"/>
       <c r="S76" s="57"/>
     </row>
     <row r="77" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3734,110 +3716,6 @@
     </row>
   </sheetData>
   <mergeCells count="118">
-    <mergeCell ref="J68:L68"/>
-    <mergeCell ref="A70:S70"/>
-    <mergeCell ref="I72:M72"/>
-    <mergeCell ref="D73:G73"/>
-    <mergeCell ref="J73:M73"/>
-    <mergeCell ref="M74:O74"/>
-    <mergeCell ref="M75:O75"/>
-    <mergeCell ref="D76:F76"/>
-    <mergeCell ref="J76:L76"/>
-    <mergeCell ref="O76:P76"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="E53:J53"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="E54:J54"/>
-    <mergeCell ref="A56:S56"/>
-    <mergeCell ref="A58:S58"/>
-    <mergeCell ref="A61:S61"/>
-    <mergeCell ref="A62:S62"/>
-    <mergeCell ref="J65:M65"/>
-    <mergeCell ref="A48:J48"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="E49:J49"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="E50:J50"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="E51:J51"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="E52:J52"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="G46:I46"/>
-    <mergeCell ref="K46:M46"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="P46:S46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="K47:M47"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="P47:S47"/>
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="G41:J41"/>
-    <mergeCell ref="K41:N41"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="G42:J42"/>
-    <mergeCell ref="K42:N42"/>
-    <mergeCell ref="A44:S44"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="K45:M45"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="P45:S45"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="G38:J38"/>
-    <mergeCell ref="K38:N38"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="G39:J39"/>
-    <mergeCell ref="K39:N39"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="G40:J40"/>
-    <mergeCell ref="K40:N40"/>
-    <mergeCell ref="A19:S19"/>
-    <mergeCell ref="A20:S20"/>
-    <mergeCell ref="A21:S21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="A34:O35"/>
-    <mergeCell ref="G36:J36"/>
-    <mergeCell ref="K36:N36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="G37:J37"/>
-    <mergeCell ref="K37:N37"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="Q15:S15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="O16:Q16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="Q17:S17"/>
-    <mergeCell ref="O11:S11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:S12"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="O13:Q13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G14:J14"/>
-    <mergeCell ref="K14:M14"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="Q14:S14"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="I11:L11"/>
-    <mergeCell ref="M11:N11"/>
     <mergeCell ref="A2:C5"/>
     <mergeCell ref="D2:P5"/>
     <mergeCell ref="Q2:S5"/>
@@ -3852,6 +3730,110 @@
     <mergeCell ref="I9:L9"/>
     <mergeCell ref="M9:O9"/>
     <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:L11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="O11:S11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:S12"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="Q14:S14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="Q15:S15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="O16:Q16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="Q17:S17"/>
+    <mergeCell ref="A19:S19"/>
+    <mergeCell ref="A20:S20"/>
+    <mergeCell ref="A21:S21"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="A34:O35"/>
+    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="K36:N36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="K37:N37"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="G38:J38"/>
+    <mergeCell ref="K38:N38"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="K39:N39"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="K40:N40"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="G41:J41"/>
+    <mergeCell ref="K41:N41"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="G42:J42"/>
+    <mergeCell ref="K42:N42"/>
+    <mergeCell ref="A44:S44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="K45:M45"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="P45:S45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="K46:M46"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="P46:S46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="P47:S47"/>
+    <mergeCell ref="A48:J48"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="E49:J49"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="E50:J50"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="E51:J51"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="E52:J52"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="E53:J53"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="E54:J54"/>
+    <mergeCell ref="A56:S56"/>
+    <mergeCell ref="A58:S58"/>
+    <mergeCell ref="A61:S61"/>
+    <mergeCell ref="A62:S62"/>
+    <mergeCell ref="J65:M65"/>
+    <mergeCell ref="J68:L68"/>
+    <mergeCell ref="A70:S70"/>
+    <mergeCell ref="I72:M72"/>
+    <mergeCell ref="D73:G73"/>
+    <mergeCell ref="J73:M73"/>
+    <mergeCell ref="M74:O74"/>
+    <mergeCell ref="M75:O75"/>
+    <mergeCell ref="D76:F76"/>
+    <mergeCell ref="J76:L76"/>
+    <mergeCell ref="O76:P76"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B23:B33" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>

<commit_message>
fix(base): desativar calculo de area base por quantidade e extrair dimensao literal do PDF
</commit_message>
<xml_diff>
--- a/public/templates/NDD-bts.xlsx
+++ b/public/templates/NDD-bts.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D3A7D15D-8C7A-44CF-B936-F320D4E0FA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D03432B-F512-458A-AFAE-85E4EEC75070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29265" yWindow="1905" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NDD" sheetId="176" r:id="rId1"/>
@@ -14,7 +14,6 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">NDD!$A1:$S77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="100">
   <si>
     <t>LOGO DETENTOR</t>
   </si>
@@ -358,13 +357,16 @@
     <t>Cargo:</t>
   </si>
   <si>
-    <t>Data da Assinatura:</t>
-  </si>
-  <si>
     <t>CLIENTE</t>
   </si>
   <si>
     <t>Pela TIM</t>
+  </si>
+  <si>
+    <t>Data da Assinatura Detentora:</t>
+  </si>
+  <si>
+    <t>Data da Assinatura TIM:</t>
   </si>
 </sst>
 </file>
@@ -1024,7 +1026,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="205">
+  <cellXfs count="206">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1200,6 +1202,306 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1290,311 +1592,14 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2031,118 +2036,118 @@
   <sheetData>
     <row r="1" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="173" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="79" t="s">
+      <c r="B2" s="174"/>
+      <c r="C2" s="174"/>
+      <c r="D2" s="179" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="79"/>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="79"/>
-      <c r="P2" s="80"/>
-      <c r="Q2" s="85"/>
-      <c r="R2" s="86"/>
-      <c r="S2" s="87"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
+      <c r="L2" s="179"/>
+      <c r="M2" s="179"/>
+      <c r="N2" s="179"/>
+      <c r="O2" s="179"/>
+      <c r="P2" s="180"/>
+      <c r="Q2" s="185"/>
+      <c r="R2" s="186"/>
+      <c r="S2" s="187"/>
       <c r="U2" t="str">
         <f t="array" aca="1" ref="U2" ca="1">CELL("nome.arquivo")</f>
         <v>C:\Users\ValtemirJunior\Downloads\NDD - Forge\public\templates\[NDD-bts.xlsx]NDD</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75"/>
-      <c r="B3" s="76"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="81"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="88"/>
-      <c r="R3" s="89"/>
-      <c r="S3" s="90"/>
+      <c r="A3" s="175"/>
+      <c r="B3" s="176"/>
+      <c r="C3" s="176"/>
+      <c r="D3" s="181"/>
+      <c r="E3" s="181"/>
+      <c r="F3" s="181"/>
+      <c r="G3" s="181"/>
+      <c r="H3" s="181"/>
+      <c r="I3" s="181"/>
+      <c r="J3" s="181"/>
+      <c r="K3" s="181"/>
+      <c r="L3" s="181"/>
+      <c r="M3" s="181"/>
+      <c r="N3" s="181"/>
+      <c r="O3" s="181"/>
+      <c r="P3" s="182"/>
+      <c r="Q3" s="188"/>
+      <c r="R3" s="189"/>
+      <c r="S3" s="190"/>
       <c r="U3" t="e">
         <f ca="1">MID(U2,FIND("WINITY_",U2)+7,FIND("_MT",U2)-FIND("WINITY_",U2)-7)</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="81"/>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
-      <c r="G4" s="81"/>
-      <c r="H4" s="81"/>
-      <c r="I4" s="81"/>
-      <c r="J4" s="81"/>
-      <c r="K4" s="81"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="81"/>
-      <c r="N4" s="81"/>
-      <c r="O4" s="81"/>
-      <c r="P4" s="82"/>
-      <c r="Q4" s="88"/>
-      <c r="R4" s="89"/>
-      <c r="S4" s="90"/>
+      <c r="A4" s="175"/>
+      <c r="B4" s="176"/>
+      <c r="C4" s="176"/>
+      <c r="D4" s="181"/>
+      <c r="E4" s="181"/>
+      <c r="F4" s="181"/>
+      <c r="G4" s="181"/>
+      <c r="H4" s="181"/>
+      <c r="I4" s="181"/>
+      <c r="J4" s="181"/>
+      <c r="K4" s="181"/>
+      <c r="L4" s="181"/>
+      <c r="M4" s="181"/>
+      <c r="N4" s="181"/>
+      <c r="O4" s="181"/>
+      <c r="P4" s="182"/>
+      <c r="Q4" s="188"/>
+      <c r="R4" s="189"/>
+      <c r="S4" s="190"/>
       <c r="U4" t="e">
         <f ca="1">TRIM(U3)</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="77"/>
-      <c r="B5" s="78"/>
-      <c r="C5" s="78"/>
-      <c r="D5" s="83"/>
-      <c r="E5" s="83"/>
-      <c r="F5" s="83"/>
-      <c r="G5" s="83"/>
-      <c r="H5" s="83"/>
-      <c r="I5" s="83"/>
-      <c r="J5" s="83"/>
-      <c r="K5" s="83"/>
-      <c r="L5" s="83"/>
-      <c r="M5" s="83"/>
-      <c r="N5" s="83"/>
-      <c r="O5" s="83"/>
-      <c r="P5" s="84"/>
-      <c r="Q5" s="91"/>
-      <c r="R5" s="92"/>
-      <c r="S5" s="93"/>
+      <c r="A5" s="177"/>
+      <c r="B5" s="178"/>
+      <c r="C5" s="178"/>
+      <c r="D5" s="183"/>
+      <c r="E5" s="183"/>
+      <c r="F5" s="183"/>
+      <c r="G5" s="183"/>
+      <c r="H5" s="183"/>
+      <c r="I5" s="183"/>
+      <c r="J5" s="183"/>
+      <c r="K5" s="183"/>
+      <c r="L5" s="183"/>
+      <c r="M5" s="183"/>
+      <c r="N5" s="183"/>
+      <c r="O5" s="183"/>
+      <c r="P5" s="184"/>
+      <c r="Q5" s="191"/>
+      <c r="R5" s="192"/>
+      <c r="S5" s="193"/>
     </row>
     <row r="6" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="94" t="s">
+      <c r="A6" s="194" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="95"/>
-      <c r="C6" s="95"/>
+      <c r="B6" s="195"/>
+      <c r="C6" s="195"/>
       <c r="D6" s="2"/>
       <c r="E6" s="3"/>
-      <c r="F6" s="96"/>
-      <c r="G6" s="96"/>
-      <c r="H6" s="96"/>
-      <c r="I6" s="96"/>
-      <c r="J6" s="96"/>
+      <c r="F6" s="196"/>
+      <c r="G6" s="196"/>
+      <c r="H6" s="196"/>
+      <c r="I6" s="196"/>
+      <c r="J6" s="196"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
@@ -2154,18 +2159,18 @@
       <c r="S6" s="5"/>
     </row>
     <row r="7" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="97" t="s">
+      <c r="A7" s="197" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="98"/>
-      <c r="C7" s="98"/>
+      <c r="B7" s="198"/>
+      <c r="C7" s="198"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="99"/>
-      <c r="G7" s="99"/>
-      <c r="H7" s="99"/>
-      <c r="I7" s="99"/>
-      <c r="J7" s="99"/>
+      <c r="F7" s="199"/>
+      <c r="G7" s="199"/>
+      <c r="H7" s="199"/>
+      <c r="I7" s="199"/>
+      <c r="J7" s="199"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
@@ -2177,74 +2182,74 @@
       <c r="S7" s="7"/>
     </row>
     <row r="8" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="100" t="s">
+      <c r="A8" s="200" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="101"/>
-      <c r="C8" s="101"/>
-      <c r="D8" s="101"/>
-      <c r="E8" s="101"/>
-      <c r="F8" s="101"/>
-      <c r="G8" s="101"/>
-      <c r="H8" s="101"/>
-      <c r="I8" s="101"/>
-      <c r="J8" s="101"/>
-      <c r="K8" s="101"/>
-      <c r="L8" s="101"/>
-      <c r="M8" s="101"/>
-      <c r="N8" s="101"/>
-      <c r="O8" s="101"/>
-      <c r="P8" s="101"/>
-      <c r="Q8" s="101"/>
-      <c r="R8" s="101"/>
-      <c r="S8" s="102"/>
+      <c r="B8" s="201"/>
+      <c r="C8" s="201"/>
+      <c r="D8" s="201"/>
+      <c r="E8" s="201"/>
+      <c r="F8" s="201"/>
+      <c r="G8" s="201"/>
+      <c r="H8" s="201"/>
+      <c r="I8" s="201"/>
+      <c r="J8" s="201"/>
+      <c r="K8" s="201"/>
+      <c r="L8" s="201"/>
+      <c r="M8" s="201"/>
+      <c r="N8" s="201"/>
+      <c r="O8" s="201"/>
+      <c r="P8" s="201"/>
+      <c r="Q8" s="201"/>
+      <c r="R8" s="201"/>
+      <c r="S8" s="202"/>
     </row>
     <row r="9" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="103" t="s">
+      <c r="A9" s="155" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="104"/>
-      <c r="C9" s="105"/>
-      <c r="D9" s="106"/>
+      <c r="B9" s="165"/>
+      <c r="C9" s="203"/>
+      <c r="D9" s="156"/>
       <c r="E9" s="9"/>
       <c r="F9" s="10"/>
-      <c r="G9" s="107" t="s">
+      <c r="G9" s="167" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="106"/>
-      <c r="I9" s="108"/>
-      <c r="J9" s="108"/>
-      <c r="K9" s="108"/>
-      <c r="L9" s="109"/>
-      <c r="M9" s="110" t="s">
+      <c r="H9" s="156"/>
+      <c r="I9" s="158"/>
+      <c r="J9" s="158"/>
+      <c r="K9" s="158"/>
+      <c r="L9" s="166"/>
+      <c r="M9" s="168" t="s">
         <v>7</v>
       </c>
-      <c r="N9" s="111"/>
-      <c r="O9" s="112"/>
-      <c r="P9" s="107"/>
-      <c r="Q9" s="106"/>
+      <c r="N9" s="169"/>
+      <c r="O9" s="204"/>
+      <c r="P9" s="167"/>
+      <c r="Q9" s="156"/>
       <c r="R9" s="11"/>
       <c r="S9" s="12"/>
     </row>
     <row r="10" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="103" t="s">
+      <c r="A10" s="155" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="106"/>
-      <c r="C10" s="106"/>
-      <c r="D10" s="106"/>
-      <c r="E10" s="106"/>
-      <c r="F10" s="106"/>
-      <c r="G10" s="104"/>
-      <c r="H10" s="107" t="s">
+      <c r="B10" s="156"/>
+      <c r="C10" s="156"/>
+      <c r="D10" s="156"/>
+      <c r="E10" s="156"/>
+      <c r="F10" s="156"/>
+      <c r="G10" s="165"/>
+      <c r="H10" s="167" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="106"/>
-      <c r="J10" s="106" t="s">
+      <c r="I10" s="156"/>
+      <c r="J10" s="156" t="s">
         <v>10</v>
       </c>
-      <c r="K10" s="106"/>
-      <c r="L10" s="106"/>
+      <c r="K10" s="156"/>
+      <c r="L10" s="156"/>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
       <c r="O10" s="9"/>
@@ -2254,67 +2259,67 @@
       <c r="S10" s="14"/>
     </row>
     <row r="11" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="103" t="s">
+      <c r="A11" s="155" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="106"/>
-      <c r="C11" s="108"/>
-      <c r="D11" s="108"/>
-      <c r="E11" s="108"/>
-      <c r="F11" s="109"/>
-      <c r="G11" s="107" t="s">
+      <c r="B11" s="156"/>
+      <c r="C11" s="158"/>
+      <c r="D11" s="158"/>
+      <c r="E11" s="158"/>
+      <c r="F11" s="166"/>
+      <c r="G11" s="167" t="s">
         <v>12</v>
       </c>
-      <c r="H11" s="106"/>
-      <c r="I11" s="108"/>
-      <c r="J11" s="108"/>
-      <c r="K11" s="108"/>
-      <c r="L11" s="109"/>
-      <c r="M11" s="113" t="s">
+      <c r="H11" s="156"/>
+      <c r="I11" s="158"/>
+      <c r="J11" s="158"/>
+      <c r="K11" s="158"/>
+      <c r="L11" s="166"/>
+      <c r="M11" s="171" t="s">
         <v>13</v>
       </c>
-      <c r="N11" s="114"/>
-      <c r="O11" s="106" t="s">
+      <c r="N11" s="172"/>
+      <c r="O11" s="156" t="s">
         <v>14</v>
       </c>
-      <c r="P11" s="106"/>
-      <c r="Q11" s="106"/>
-      <c r="R11" s="106"/>
-      <c r="S11" s="115"/>
+      <c r="P11" s="156"/>
+      <c r="Q11" s="156"/>
+      <c r="R11" s="156"/>
+      <c r="S11" s="163"/>
     </row>
     <row r="12" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="103" t="s">
+      <c r="A12" s="155" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="106"/>
-      <c r="C12" s="106"/>
-      <c r="D12" s="116"/>
-      <c r="E12" s="106"/>
-      <c r="F12" s="106"/>
-      <c r="G12" s="106"/>
-      <c r="H12" s="106"/>
-      <c r="I12" s="106"/>
-      <c r="J12" s="106"/>
-      <c r="K12" s="106"/>
-      <c r="L12" s="106"/>
-      <c r="M12" s="106"/>
-      <c r="N12" s="106"/>
-      <c r="O12" s="106"/>
-      <c r="P12" s="106"/>
-      <c r="Q12" s="106"/>
-      <c r="R12" s="106"/>
-      <c r="S12" s="115"/>
+      <c r="B12" s="156"/>
+      <c r="C12" s="156"/>
+      <c r="D12" s="164"/>
+      <c r="E12" s="156"/>
+      <c r="F12" s="156"/>
+      <c r="G12" s="156"/>
+      <c r="H12" s="156"/>
+      <c r="I12" s="156"/>
+      <c r="J12" s="156"/>
+      <c r="K12" s="156"/>
+      <c r="L12" s="156"/>
+      <c r="M12" s="156"/>
+      <c r="N12" s="156"/>
+      <c r="O12" s="156"/>
+      <c r="P12" s="156"/>
+      <c r="Q12" s="156"/>
+      <c r="R12" s="156"/>
+      <c r="S12" s="163"/>
     </row>
     <row r="13" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="106"/>
-      <c r="C13" s="106"/>
-      <c r="D13" s="106"/>
-      <c r="E13" s="106"/>
-      <c r="F13" s="106"/>
-      <c r="G13" s="104"/>
+      <c r="B13" s="156"/>
+      <c r="C13" s="156"/>
+      <c r="D13" s="156"/>
+      <c r="E13" s="156"/>
+      <c r="F13" s="156"/>
+      <c r="G13" s="165"/>
       <c r="H13" s="16" t="s">
         <v>17</v>
       </c>
@@ -2326,89 +2331,89 @@
       <c r="N13" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="O13" s="108"/>
-      <c r="P13" s="108"/>
-      <c r="Q13" s="109"/>
+      <c r="O13" s="158"/>
+      <c r="P13" s="158"/>
+      <c r="Q13" s="166"/>
       <c r="R13" s="18" t="s">
         <v>19</v>
       </c>
       <c r="S13" s="14"/>
     </row>
     <row r="14" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="103" t="s">
+      <c r="A14" s="155" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="106"/>
-      <c r="C14" s="106"/>
-      <c r="D14" s="108"/>
-      <c r="E14" s="108"/>
-      <c r="F14" s="109"/>
-      <c r="G14" s="107" t="s">
+      <c r="B14" s="156"/>
+      <c r="C14" s="156"/>
+      <c r="D14" s="158"/>
+      <c r="E14" s="158"/>
+      <c r="F14" s="166"/>
+      <c r="G14" s="167" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="106"/>
-      <c r="I14" s="106"/>
-      <c r="J14" s="106"/>
-      <c r="K14" s="106" t="s">
+      <c r="H14" s="156"/>
+      <c r="I14" s="156"/>
+      <c r="J14" s="156"/>
+      <c r="K14" s="156" t="s">
         <v>14</v>
       </c>
-      <c r="L14" s="106"/>
-      <c r="M14" s="104"/>
-      <c r="N14" s="110" t="s">
+      <c r="L14" s="156"/>
+      <c r="M14" s="165"/>
+      <c r="N14" s="168" t="s">
         <v>22</v>
       </c>
-      <c r="O14" s="111"/>
-      <c r="P14" s="111"/>
-      <c r="Q14" s="111" t="s">
+      <c r="O14" s="169"/>
+      <c r="P14" s="169"/>
+      <c r="Q14" s="169" t="s">
         <v>14</v>
       </c>
-      <c r="R14" s="111"/>
-      <c r="S14" s="117"/>
+      <c r="R14" s="169"/>
+      <c r="S14" s="170"/>
     </row>
     <row r="15" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="103" t="s">
+      <c r="A15" s="155" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="106"/>
-      <c r="C15" s="106"/>
+      <c r="B15" s="156"/>
+      <c r="C15" s="156"/>
       <c r="D15" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="106" t="s">
+      <c r="E15" s="156" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="106"/>
+      <c r="F15" s="156"/>
       <c r="G15" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="H15" s="106" t="s">
+      <c r="H15" s="156" t="s">
         <v>27</v>
       </c>
-      <c r="I15" s="106"/>
+      <c r="I15" s="156"/>
       <c r="J15" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="K15" s="118" t="s">
+      <c r="K15" s="157" t="s">
         <v>29</v>
       </c>
-      <c r="L15" s="118"/>
+      <c r="L15" s="157"/>
       <c r="M15" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="N15" s="108" t="s">
+      <c r="N15" s="158" t="s">
         <v>31</v>
       </c>
-      <c r="O15" s="108"/>
-      <c r="P15" s="108"/>
-      <c r="Q15" s="119"/>
-      <c r="R15" s="119"/>
-      <c r="S15" s="120"/>
+      <c r="O15" s="158"/>
+      <c r="P15" s="158"/>
+      <c r="Q15" s="159"/>
+      <c r="R15" s="159"/>
+      <c r="S15" s="160"/>
     </row>
     <row r="16" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="103" t="s">
+      <c r="A16" s="155" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="106"/>
+      <c r="B16" s="156"/>
       <c r="C16" s="19" t="s">
         <v>33</v>
       </c>
@@ -2443,19 +2448,19 @@
       <c r="N16" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="O16" s="108" t="s">
+      <c r="O16" s="158" t="s">
         <v>31</v>
       </c>
-      <c r="P16" s="108"/>
-      <c r="Q16" s="108"/>
+      <c r="P16" s="158"/>
+      <c r="Q16" s="158"/>
       <c r="R16" s="13"/>
       <c r="S16" s="20"/>
     </row>
     <row r="17" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="121" t="s">
+      <c r="A17" s="161" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="122"/>
+      <c r="B17" s="162"/>
       <c r="C17" s="19" t="s">
         <v>35</v>
       </c>
@@ -2473,10 +2478,10 @@
       <c r="I17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J17" s="118" t="s">
+      <c r="J17" s="157" t="s">
         <v>43</v>
       </c>
-      <c r="K17" s="118"/>
+      <c r="K17" s="157"/>
       <c r="L17" s="4"/>
       <c r="M17" s="1" t="s">
         <v>44</v>
@@ -2488,11 +2493,11 @@
       <c r="P17" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="Q17" s="106" t="s">
+      <c r="Q17" s="156" t="s">
         <v>31</v>
       </c>
-      <c r="R17" s="106"/>
-      <c r="S17" s="115"/>
+      <c r="R17" s="156"/>
+      <c r="S17" s="163"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="22"/>
@@ -2513,73 +2518,73 @@
       <c r="S18" s="31"/>
     </row>
     <row r="19" spans="1:19" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="123" t="s">
+      <c r="A19" s="88" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
-      <c r="F19" s="124"/>
-      <c r="G19" s="124"/>
-      <c r="H19" s="124"/>
-      <c r="I19" s="124"/>
-      <c r="J19" s="124"/>
-      <c r="K19" s="124"/>
-      <c r="L19" s="124"/>
-      <c r="M19" s="124"/>
-      <c r="N19" s="124"/>
-      <c r="O19" s="124"/>
-      <c r="P19" s="124"/>
-      <c r="Q19" s="124"/>
-      <c r="R19" s="124"/>
-      <c r="S19" s="125"/>
+      <c r="B19" s="89"/>
+      <c r="C19" s="89"/>
+      <c r="D19" s="89"/>
+      <c r="E19" s="89"/>
+      <c r="F19" s="89"/>
+      <c r="G19" s="89"/>
+      <c r="H19" s="89"/>
+      <c r="I19" s="89"/>
+      <c r="J19" s="89"/>
+      <c r="K19" s="89"/>
+      <c r="L19" s="89"/>
+      <c r="M19" s="89"/>
+      <c r="N19" s="89"/>
+      <c r="O19" s="89"/>
+      <c r="P19" s="89"/>
+      <c r="Q19" s="89"/>
+      <c r="R19" s="89"/>
+      <c r="S19" s="90"/>
     </row>
     <row r="20" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="126" t="s">
+      <c r="A20" s="138" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="127"/>
-      <c r="C20" s="127"/>
-      <c r="D20" s="127"/>
-      <c r="E20" s="127"/>
-      <c r="F20" s="127"/>
-      <c r="G20" s="127"/>
-      <c r="H20" s="127"/>
-      <c r="I20" s="127"/>
-      <c r="J20" s="127"/>
-      <c r="K20" s="127"/>
-      <c r="L20" s="127"/>
-      <c r="M20" s="127"/>
-      <c r="N20" s="127"/>
-      <c r="O20" s="127"/>
-      <c r="P20" s="127"/>
-      <c r="Q20" s="127"/>
-      <c r="R20" s="127"/>
-      <c r="S20" s="128"/>
+      <c r="B20" s="139"/>
+      <c r="C20" s="139"/>
+      <c r="D20" s="139"/>
+      <c r="E20" s="139"/>
+      <c r="F20" s="139"/>
+      <c r="G20" s="139"/>
+      <c r="H20" s="139"/>
+      <c r="I20" s="139"/>
+      <c r="J20" s="139"/>
+      <c r="K20" s="139"/>
+      <c r="L20" s="139"/>
+      <c r="M20" s="139"/>
+      <c r="N20" s="139"/>
+      <c r="O20" s="139"/>
+      <c r="P20" s="139"/>
+      <c r="Q20" s="139"/>
+      <c r="R20" s="139"/>
+      <c r="S20" s="140"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="129" t="s">
+      <c r="A21" s="121" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="130"/>
-      <c r="C21" s="130"/>
-      <c r="D21" s="130"/>
-      <c r="E21" s="130"/>
-      <c r="F21" s="130"/>
-      <c r="G21" s="130"/>
-      <c r="H21" s="130"/>
-      <c r="I21" s="130"/>
-      <c r="J21" s="130"/>
-      <c r="K21" s="130"/>
-      <c r="L21" s="130"/>
-      <c r="M21" s="130"/>
-      <c r="N21" s="130"/>
-      <c r="O21" s="130"/>
-      <c r="P21" s="130"/>
-      <c r="Q21" s="130"/>
-      <c r="R21" s="130"/>
-      <c r="S21" s="131"/>
+      <c r="B21" s="122"/>
+      <c r="C21" s="122"/>
+      <c r="D21" s="122"/>
+      <c r="E21" s="122"/>
+      <c r="F21" s="122"/>
+      <c r="G21" s="122"/>
+      <c r="H21" s="122"/>
+      <c r="I21" s="122"/>
+      <c r="J21" s="122"/>
+      <c r="K21" s="122"/>
+      <c r="L21" s="122"/>
+      <c r="M21" s="122"/>
+      <c r="N21" s="122"/>
+      <c r="O21" s="122"/>
+      <c r="P21" s="122"/>
+      <c r="Q21" s="122"/>
+      <c r="R21" s="122"/>
+      <c r="S21" s="123"/>
     </row>
     <row r="22" spans="1:19" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
@@ -2594,10 +2599,10 @@
       <c r="D22" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="132" t="s">
+      <c r="E22" s="141" t="s">
         <v>54</v>
       </c>
-      <c r="F22" s="133"/>
+      <c r="F22" s="142"/>
       <c r="G22" s="33" t="s">
         <v>55</v>
       </c>
@@ -2631,10 +2636,10 @@
       <c r="Q22" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="R22" s="132" t="s">
+      <c r="R22" s="141" t="s">
         <v>66</v>
       </c>
-      <c r="S22" s="134"/>
+      <c r="S22" s="143"/>
     </row>
     <row r="23" spans="1:19" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="34"/>
@@ -2868,23 +2873,23 @@
       <c r="S33" s="41"/>
     </row>
     <row r="34" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="135" t="s">
+      <c r="A34" s="144" t="s">
         <v>67</v>
       </c>
-      <c r="B34" s="136"/>
-      <c r="C34" s="136"/>
-      <c r="D34" s="136"/>
-      <c r="E34" s="136"/>
-      <c r="F34" s="136"/>
-      <c r="G34" s="136"/>
-      <c r="H34" s="136"/>
-      <c r="I34" s="136"/>
-      <c r="J34" s="136"/>
-      <c r="K34" s="136"/>
-      <c r="L34" s="136"/>
-      <c r="M34" s="136"/>
-      <c r="N34" s="136"/>
-      <c r="O34" s="136"/>
+      <c r="B34" s="145"/>
+      <c r="C34" s="145"/>
+      <c r="D34" s="145"/>
+      <c r="E34" s="145"/>
+      <c r="F34" s="145"/>
+      <c r="G34" s="145"/>
+      <c r="H34" s="145"/>
+      <c r="I34" s="145"/>
+      <c r="J34" s="145"/>
+      <c r="K34" s="145"/>
+      <c r="L34" s="145"/>
+      <c r="M34" s="145"/>
+      <c r="N34" s="145"/>
+      <c r="O34" s="145"/>
       <c r="P34" s="45"/>
       <c r="Q34" s="45"/>
       <c r="R34" s="45"/>
@@ -2892,21 +2897,21 @@
       <c r="T34" s="47"/>
     </row>
     <row r="35" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="137"/>
-      <c r="B35" s="138"/>
-      <c r="C35" s="138"/>
-      <c r="D35" s="138"/>
-      <c r="E35" s="138"/>
-      <c r="F35" s="138"/>
-      <c r="G35" s="138"/>
-      <c r="H35" s="138"/>
-      <c r="I35" s="138"/>
-      <c r="J35" s="138"/>
-      <c r="K35" s="138"/>
-      <c r="L35" s="138"/>
-      <c r="M35" s="138"/>
-      <c r="N35" s="138"/>
-      <c r="O35" s="138"/>
+      <c r="A35" s="146"/>
+      <c r="B35" s="147"/>
+      <c r="C35" s="147"/>
+      <c r="D35" s="147"/>
+      <c r="E35" s="147"/>
+      <c r="F35" s="147"/>
+      <c r="G35" s="147"/>
+      <c r="H35" s="147"/>
+      <c r="I35" s="147"/>
+      <c r="J35" s="147"/>
+      <c r="K35" s="147"/>
+      <c r="L35" s="147"/>
+      <c r="M35" s="147"/>
+      <c r="N35" s="147"/>
+      <c r="O35" s="147"/>
       <c r="S35" s="48"/>
       <c r="T35" s="47"/>
     </row>
@@ -2917,18 +2922,18 @@
       <c r="D36" s="50"/>
       <c r="E36" s="50"/>
       <c r="F36" s="50"/>
-      <c r="G36" s="139" t="s">
+      <c r="G36" s="148" t="s">
         <v>68</v>
       </c>
-      <c r="H36" s="140"/>
-      <c r="I36" s="140"/>
-      <c r="J36" s="141"/>
-      <c r="K36" s="139" t="s">
+      <c r="H36" s="149"/>
+      <c r="I36" s="149"/>
+      <c r="J36" s="150"/>
+      <c r="K36" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="L36" s="140"/>
-      <c r="M36" s="140"/>
-      <c r="N36" s="141"/>
+      <c r="L36" s="149"/>
+      <c r="M36" s="149"/>
+      <c r="N36" s="150"/>
       <c r="O36" s="47"/>
       <c r="P36" s="47"/>
       <c r="Q36" s="47"/>
@@ -2937,22 +2942,22 @@
       <c r="T36" s="47"/>
     </row>
     <row r="37" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="142" t="s">
+      <c r="A37" s="151" t="s">
         <v>70</v>
       </c>
-      <c r="B37" s="143"/>
-      <c r="C37" s="143"/>
-      <c r="D37" s="143"/>
-      <c r="E37" s="143"/>
-      <c r="F37" s="144"/>
-      <c r="G37" s="145"/>
-      <c r="H37" s="146"/>
-      <c r="I37" s="146"/>
-      <c r="J37" s="147"/>
-      <c r="K37" s="148"/>
-      <c r="L37" s="149"/>
-      <c r="M37" s="149"/>
-      <c r="N37" s="150"/>
+      <c r="B37" s="112"/>
+      <c r="C37" s="112"/>
+      <c r="D37" s="112"/>
+      <c r="E37" s="112"/>
+      <c r="F37" s="113"/>
+      <c r="G37" s="118"/>
+      <c r="H37" s="119"/>
+      <c r="I37" s="119"/>
+      <c r="J37" s="120"/>
+      <c r="K37" s="152"/>
+      <c r="L37" s="153"/>
+      <c r="M37" s="153"/>
+      <c r="N37" s="154"/>
       <c r="O37" s="47"/>
       <c r="P37" s="47"/>
       <c r="Q37" s="47"/>
@@ -2960,22 +2965,22 @@
       <c r="S37" s="51"/>
     </row>
     <row r="38" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="151" t="s">
+      <c r="A38" s="111" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="143"/>
-      <c r="C38" s="143"/>
-      <c r="D38" s="143"/>
-      <c r="E38" s="143"/>
-      <c r="F38" s="144"/>
-      <c r="G38" s="145"/>
-      <c r="H38" s="146"/>
-      <c r="I38" s="146"/>
-      <c r="J38" s="147"/>
-      <c r="K38" s="145"/>
-      <c r="L38" s="146"/>
-      <c r="M38" s="146"/>
-      <c r="N38" s="147"/>
+      <c r="B38" s="112"/>
+      <c r="C38" s="112"/>
+      <c r="D38" s="112"/>
+      <c r="E38" s="112"/>
+      <c r="F38" s="113"/>
+      <c r="G38" s="118"/>
+      <c r="H38" s="119"/>
+      <c r="I38" s="119"/>
+      <c r="J38" s="120"/>
+      <c r="K38" s="118"/>
+      <c r="L38" s="119"/>
+      <c r="M38" s="119"/>
+      <c r="N38" s="120"/>
       <c r="O38" s="47"/>
       <c r="P38" s="47"/>
       <c r="Q38" s="47"/>
@@ -2983,22 +2988,22 @@
       <c r="S38" s="51"/>
     </row>
     <row r="39" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="152" t="s">
+      <c r="A39" s="132" t="s">
         <v>72</v>
       </c>
-      <c r="B39" s="153"/>
-      <c r="C39" s="153"/>
-      <c r="D39" s="153"/>
-      <c r="E39" s="153"/>
-      <c r="F39" s="154"/>
-      <c r="G39" s="145"/>
-      <c r="H39" s="146"/>
-      <c r="I39" s="146"/>
-      <c r="J39" s="147"/>
-      <c r="K39" s="145"/>
-      <c r="L39" s="146"/>
-      <c r="M39" s="146"/>
-      <c r="N39" s="147"/>
+      <c r="B39" s="133"/>
+      <c r="C39" s="133"/>
+      <c r="D39" s="133"/>
+      <c r="E39" s="133"/>
+      <c r="F39" s="134"/>
+      <c r="G39" s="118"/>
+      <c r="H39" s="119"/>
+      <c r="I39" s="119"/>
+      <c r="J39" s="120"/>
+      <c r="K39" s="118"/>
+      <c r="L39" s="119"/>
+      <c r="M39" s="119"/>
+      <c r="N39" s="120"/>
       <c r="O39" s="47"/>
       <c r="P39" s="47"/>
       <c r="Q39" s="47"/>
@@ -3006,26 +3011,26 @@
       <c r="S39" s="51"/>
     </row>
     <row r="40" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="155" t="s">
+      <c r="A40" s="135" t="s">
         <v>73</v>
       </c>
-      <c r="B40" s="156"/>
-      <c r="C40" s="156"/>
-      <c r="D40" s="156"/>
-      <c r="E40" s="156"/>
-      <c r="F40" s="157"/>
-      <c r="G40" s="158" t="s">
+      <c r="B40" s="136"/>
+      <c r="C40" s="136"/>
+      <c r="D40" s="136"/>
+      <c r="E40" s="136"/>
+      <c r="F40" s="137"/>
+      <c r="G40" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="H40" s="159"/>
-      <c r="I40" s="159"/>
-      <c r="J40" s="160"/>
-      <c r="K40" s="158" t="s">
+      <c r="H40" s="98"/>
+      <c r="I40" s="98"/>
+      <c r="J40" s="99"/>
+      <c r="K40" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="L40" s="159"/>
-      <c r="M40" s="159"/>
-      <c r="N40" s="160"/>
+      <c r="L40" s="98"/>
+      <c r="M40" s="98"/>
+      <c r="N40" s="99"/>
       <c r="O40" s="47"/>
       <c r="P40" s="47"/>
       <c r="Q40" s="47"/>
@@ -3033,26 +3038,26 @@
       <c r="S40" s="51"/>
     </row>
     <row r="41" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="151" t="s">
+      <c r="A41" s="111" t="s">
         <v>74</v>
       </c>
-      <c r="B41" s="143"/>
-      <c r="C41" s="143"/>
-      <c r="D41" s="143"/>
-      <c r="E41" s="143"/>
-      <c r="F41" s="144"/>
-      <c r="G41" s="158" t="s">
+      <c r="B41" s="112"/>
+      <c r="C41" s="112"/>
+      <c r="D41" s="112"/>
+      <c r="E41" s="112"/>
+      <c r="F41" s="113"/>
+      <c r="G41" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="H41" s="159"/>
-      <c r="I41" s="159"/>
-      <c r="J41" s="160"/>
-      <c r="K41" s="158" t="s">
+      <c r="H41" s="98"/>
+      <c r="I41" s="98"/>
+      <c r="J41" s="99"/>
+      <c r="K41" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="L41" s="159"/>
-      <c r="M41" s="159"/>
-      <c r="N41" s="160"/>
+      <c r="L41" s="98"/>
+      <c r="M41" s="98"/>
+      <c r="N41" s="99"/>
       <c r="O41" s="47"/>
       <c r="P41" s="47"/>
       <c r="Q41" s="47"/>
@@ -3060,28 +3065,28 @@
       <c r="S41" s="51"/>
     </row>
     <row r="42" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="161" t="s">
+      <c r="A42" s="115" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="162"/>
-      <c r="C42" s="162"/>
-      <c r="D42" s="162"/>
-      <c r="E42" s="162"/>
-      <c r="F42" s="163"/>
-      <c r="G42" s="145">
+      <c r="B42" s="116"/>
+      <c r="C42" s="116"/>
+      <c r="D42" s="116"/>
+      <c r="E42" s="116"/>
+      <c r="F42" s="117"/>
+      <c r="G42" s="118">
         <f>G37</f>
         <v>0</v>
       </c>
-      <c r="H42" s="146"/>
-      <c r="I42" s="146"/>
-      <c r="J42" s="147"/>
-      <c r="K42" s="145">
+      <c r="H42" s="119"/>
+      <c r="I42" s="119"/>
+      <c r="J42" s="120"/>
+      <c r="K42" s="118">
         <f>K37</f>
         <v>0</v>
       </c>
-      <c r="L42" s="159"/>
-      <c r="M42" s="159"/>
-      <c r="N42" s="160"/>
+      <c r="L42" s="98"/>
+      <c r="M42" s="98"/>
+      <c r="N42" s="99"/>
       <c r="O42" s="47"/>
       <c r="P42" s="47"/>
       <c r="Q42" s="47"/>
@@ -3110,144 +3115,144 @@
       <c r="S43" s="54"/>
     </row>
     <row r="44" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="129" t="s">
+      <c r="A44" s="121" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="130"/>
-      <c r="C44" s="130"/>
-      <c r="D44" s="130"/>
-      <c r="E44" s="130"/>
-      <c r="F44" s="130"/>
-      <c r="G44" s="130"/>
-      <c r="H44" s="130"/>
-      <c r="I44" s="130"/>
-      <c r="J44" s="130"/>
-      <c r="K44" s="130"/>
-      <c r="L44" s="130"/>
-      <c r="M44" s="130"/>
-      <c r="N44" s="130"/>
-      <c r="O44" s="130"/>
-      <c r="P44" s="130"/>
-      <c r="Q44" s="130"/>
-      <c r="R44" s="130"/>
-      <c r="S44" s="131"/>
+      <c r="B44" s="122"/>
+      <c r="C44" s="122"/>
+      <c r="D44" s="122"/>
+      <c r="E44" s="122"/>
+      <c r="F44" s="122"/>
+      <c r="G44" s="122"/>
+      <c r="H44" s="122"/>
+      <c r="I44" s="122"/>
+      <c r="J44" s="122"/>
+      <c r="K44" s="122"/>
+      <c r="L44" s="122"/>
+      <c r="M44" s="122"/>
+      <c r="N44" s="122"/>
+      <c r="O44" s="122"/>
+      <c r="P44" s="122"/>
+      <c r="Q44" s="122"/>
+      <c r="R44" s="122"/>
+      <c r="S44" s="123"/>
     </row>
     <row r="45" spans="1:20" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="164" t="s">
+      <c r="A45" s="124" t="s">
         <v>51</v>
       </c>
-      <c r="B45" s="165"/>
-      <c r="C45" s="166"/>
-      <c r="D45" s="167" t="s">
+      <c r="B45" s="125"/>
+      <c r="C45" s="126"/>
+      <c r="D45" s="127" t="s">
         <v>53</v>
       </c>
-      <c r="E45" s="168"/>
-      <c r="F45" s="169"/>
-      <c r="G45" s="167" t="s">
+      <c r="E45" s="128"/>
+      <c r="F45" s="129"/>
+      <c r="G45" s="127" t="s">
         <v>54</v>
       </c>
-      <c r="H45" s="168"/>
-      <c r="I45" s="169"/>
+      <c r="H45" s="128"/>
+      <c r="I45" s="129"/>
       <c r="J45" s="55" t="s">
         <v>55</v>
       </c>
-      <c r="K45" s="170" t="s">
+      <c r="K45" s="130" t="s">
         <v>77</v>
       </c>
-      <c r="L45" s="165"/>
-      <c r="M45" s="166"/>
-      <c r="N45" s="170" t="s">
+      <c r="L45" s="125"/>
+      <c r="M45" s="126"/>
+      <c r="N45" s="130" t="s">
         <v>78</v>
       </c>
-      <c r="O45" s="166"/>
-      <c r="P45" s="167" t="s">
+      <c r="O45" s="126"/>
+      <c r="P45" s="127" t="s">
         <v>66</v>
       </c>
-      <c r="Q45" s="168"/>
-      <c r="R45" s="168"/>
-      <c r="S45" s="171"/>
+      <c r="Q45" s="128"/>
+      <c r="R45" s="128"/>
+      <c r="S45" s="131"/>
     </row>
     <row r="46" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="172" t="s">
+      <c r="A46" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="B46" s="173"/>
-      <c r="C46" s="174"/>
-      <c r="D46" s="175" t="s">
+      <c r="B46" s="107"/>
+      <c r="C46" s="108"/>
+      <c r="D46" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="E46" s="173"/>
-      <c r="F46" s="174"/>
-      <c r="G46" s="175" t="s">
+      <c r="E46" s="107"/>
+      <c r="F46" s="108"/>
+      <c r="G46" s="109" t="s">
         <v>80</v>
       </c>
-      <c r="H46" s="173"/>
-      <c r="I46" s="174"/>
+      <c r="H46" s="107"/>
+      <c r="I46" s="108"/>
       <c r="J46" s="56">
         <v>1</v>
       </c>
-      <c r="K46" s="175"/>
-      <c r="L46" s="173"/>
-      <c r="M46" s="174"/>
-      <c r="N46" s="175" t="s">
+      <c r="K46" s="109"/>
+      <c r="L46" s="107"/>
+      <c r="M46" s="108"/>
+      <c r="N46" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="O46" s="174"/>
-      <c r="P46" s="175" t="s">
+      <c r="O46" s="108"/>
+      <c r="P46" s="109" t="s">
         <v>80</v>
       </c>
-      <c r="Q46" s="173"/>
-      <c r="R46" s="173"/>
-      <c r="S46" s="176"/>
+      <c r="Q46" s="107"/>
+      <c r="R46" s="107"/>
+      <c r="S46" s="110"/>
     </row>
     <row r="47" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="172" t="s">
+      <c r="A47" s="106" t="s">
         <v>79</v>
       </c>
-      <c r="B47" s="173"/>
-      <c r="C47" s="174"/>
-      <c r="D47" s="175" t="s">
+      <c r="B47" s="107"/>
+      <c r="C47" s="108"/>
+      <c r="D47" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="E47" s="173"/>
-      <c r="F47" s="174"/>
-      <c r="G47" s="175" t="s">
+      <c r="E47" s="107"/>
+      <c r="F47" s="108"/>
+      <c r="G47" s="109" t="s">
         <v>81</v>
       </c>
-      <c r="H47" s="173"/>
-      <c r="I47" s="174"/>
+      <c r="H47" s="107"/>
+      <c r="I47" s="108"/>
       <c r="J47" s="56">
         <v>1</v>
       </c>
-      <c r="K47" s="175" t="s">
+      <c r="K47" s="109" t="s">
         <v>82</v>
       </c>
-      <c r="L47" s="173"/>
-      <c r="M47" s="174"/>
-      <c r="N47" s="175" t="s">
+      <c r="L47" s="107"/>
+      <c r="M47" s="108"/>
+      <c r="N47" s="109" t="s">
         <v>14</v>
       </c>
-      <c r="O47" s="174"/>
-      <c r="P47" s="175" t="s">
+      <c r="O47" s="108"/>
+      <c r="P47" s="109" t="s">
         <v>81</v>
       </c>
-      <c r="Q47" s="173"/>
-      <c r="R47" s="173"/>
-      <c r="S47" s="176"/>
+      <c r="Q47" s="107"/>
+      <c r="R47" s="107"/>
+      <c r="S47" s="110"/>
     </row>
     <row r="48" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="177" t="s">
+      <c r="A48" s="97" t="s">
         <v>83</v>
       </c>
-      <c r="B48" s="159"/>
-      <c r="C48" s="159"/>
-      <c r="D48" s="159"/>
-      <c r="E48" s="159"/>
-      <c r="F48" s="159"/>
-      <c r="G48" s="159"/>
-      <c r="H48" s="159"/>
-      <c r="I48" s="159"/>
-      <c r="J48" s="160"/>
+      <c r="B48" s="98"/>
+      <c r="C48" s="98"/>
+      <c r="D48" s="98"/>
+      <c r="E48" s="98"/>
+      <c r="F48" s="98"/>
+      <c r="G48" s="98"/>
+      <c r="H48" s="98"/>
+      <c r="I48" s="98"/>
+      <c r="J48" s="99"/>
       <c r="K48" s="47"/>
       <c r="L48" s="47"/>
       <c r="M48" s="47"/>
@@ -3259,106 +3264,106 @@
       <c r="S48" s="52"/>
     </row>
     <row r="49" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="178" t="s">
+      <c r="A49" s="79" t="s">
         <v>84</v>
       </c>
-      <c r="B49" s="179"/>
-      <c r="C49" s="179"/>
-      <c r="D49" s="180"/>
-      <c r="E49" s="181"/>
-      <c r="F49" s="182"/>
-      <c r="G49" s="182"/>
-      <c r="H49" s="182"/>
-      <c r="I49" s="182"/>
-      <c r="J49" s="183"/>
+      <c r="B49" s="80"/>
+      <c r="C49" s="80"/>
+      <c r="D49" s="81"/>
+      <c r="E49" s="82"/>
+      <c r="F49" s="83"/>
+      <c r="G49" s="83"/>
+      <c r="H49" s="83"/>
+      <c r="I49" s="83"/>
+      <c r="J49" s="84"/>
       <c r="S49" s="57"/>
     </row>
     <row r="50" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="178" t="s">
+      <c r="A50" s="79" t="s">
         <v>85</v>
       </c>
-      <c r="B50" s="179"/>
-      <c r="C50" s="179"/>
-      <c r="D50" s="180"/>
-      <c r="E50" s="181">
+      <c r="B50" s="80"/>
+      <c r="C50" s="80"/>
+      <c r="D50" s="81"/>
+      <c r="E50" s="82">
         <f>10-E49</f>
         <v>10</v>
       </c>
-      <c r="F50" s="182"/>
-      <c r="G50" s="182"/>
-      <c r="H50" s="182"/>
-      <c r="I50" s="182"/>
-      <c r="J50" s="183"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="83"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="83"/>
+      <c r="J50" s="84"/>
       <c r="S50" s="57"/>
     </row>
     <row r="51" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="184" t="s">
+      <c r="A51" s="100" t="s">
         <v>86</v>
       </c>
-      <c r="B51" s="185"/>
-      <c r="C51" s="185"/>
-      <c r="D51" s="186"/>
-      <c r="E51" s="181">
+      <c r="B51" s="101"/>
+      <c r="C51" s="101"/>
+      <c r="D51" s="102"/>
+      <c r="E51" s="82">
         <f>E49</f>
         <v>0</v>
       </c>
-      <c r="F51" s="182"/>
-      <c r="G51" s="182"/>
-      <c r="H51" s="182"/>
-      <c r="I51" s="182"/>
-      <c r="J51" s="183"/>
+      <c r="F51" s="83"/>
+      <c r="G51" s="83"/>
+      <c r="H51" s="83"/>
+      <c r="I51" s="83"/>
+      <c r="J51" s="84"/>
       <c r="S51" s="57"/>
     </row>
     <row r="52" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="187" t="s">
+      <c r="A52" s="103" t="s">
         <v>87</v>
       </c>
-      <c r="B52" s="188"/>
-      <c r="C52" s="188"/>
-      <c r="D52" s="189"/>
-      <c r="E52" s="181" t="s">
+      <c r="B52" s="104"/>
+      <c r="C52" s="104"/>
+      <c r="D52" s="105"/>
+      <c r="E52" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="F52" s="182"/>
-      <c r="G52" s="182"/>
-      <c r="H52" s="182"/>
-      <c r="I52" s="182"/>
-      <c r="J52" s="183"/>
+      <c r="F52" s="83"/>
+      <c r="G52" s="83"/>
+      <c r="H52" s="83"/>
+      <c r="I52" s="83"/>
+      <c r="J52" s="84"/>
       <c r="S52" s="57"/>
     </row>
     <row r="53" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="178" t="s">
+      <c r="A53" s="79" t="s">
         <v>88</v>
       </c>
-      <c r="B53" s="179"/>
-      <c r="C53" s="179"/>
-      <c r="D53" s="180"/>
-      <c r="E53" s="181" t="s">
+      <c r="B53" s="80"/>
+      <c r="C53" s="80"/>
+      <c r="D53" s="81"/>
+      <c r="E53" s="82" t="s">
         <v>14</v>
       </c>
-      <c r="F53" s="182"/>
-      <c r="G53" s="182"/>
-      <c r="H53" s="182"/>
-      <c r="I53" s="182"/>
-      <c r="J53" s="183"/>
+      <c r="F53" s="83"/>
+      <c r="G53" s="83"/>
+      <c r="H53" s="83"/>
+      <c r="I53" s="83"/>
+      <c r="J53" s="84"/>
       <c r="S53" s="57"/>
     </row>
     <row r="54" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="190" t="s">
+      <c r="A54" s="85" t="s">
         <v>89</v>
       </c>
-      <c r="B54" s="191"/>
-      <c r="C54" s="191"/>
-      <c r="D54" s="192"/>
-      <c r="E54" s="181">
+      <c r="B54" s="86"/>
+      <c r="C54" s="86"/>
+      <c r="D54" s="87"/>
+      <c r="E54" s="82">
         <f>E49</f>
         <v>0</v>
       </c>
-      <c r="F54" s="182"/>
-      <c r="G54" s="182"/>
-      <c r="H54" s="182"/>
-      <c r="I54" s="182"/>
-      <c r="J54" s="183"/>
+      <c r="F54" s="83"/>
+      <c r="G54" s="83"/>
+      <c r="H54" s="83"/>
+      <c r="I54" s="83"/>
+      <c r="J54" s="84"/>
       <c r="S54" s="57"/>
     </row>
     <row r="55" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3366,54 +3371,54 @@
       <c r="S55" s="57"/>
     </row>
     <row r="56" spans="1:26" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="123" t="s">
+      <c r="A56" s="88" t="s">
         <v>66</v>
       </c>
-      <c r="B56" s="124"/>
-      <c r="C56" s="124"/>
-      <c r="D56" s="124"/>
-      <c r="E56" s="124"/>
-      <c r="F56" s="124"/>
-      <c r="G56" s="124"/>
-      <c r="H56" s="124"/>
-      <c r="I56" s="124"/>
-      <c r="J56" s="124"/>
-      <c r="K56" s="124"/>
-      <c r="L56" s="124"/>
-      <c r="M56" s="124"/>
-      <c r="N56" s="124"/>
-      <c r="O56" s="124"/>
-      <c r="P56" s="124"/>
-      <c r="Q56" s="124"/>
-      <c r="R56" s="124"/>
-      <c r="S56" s="125"/>
+      <c r="B56" s="89"/>
+      <c r="C56" s="89"/>
+      <c r="D56" s="89"/>
+      <c r="E56" s="89"/>
+      <c r="F56" s="89"/>
+      <c r="G56" s="89"/>
+      <c r="H56" s="89"/>
+      <c r="I56" s="89"/>
+      <c r="J56" s="89"/>
+      <c r="K56" s="89"/>
+      <c r="L56" s="89"/>
+      <c r="M56" s="89"/>
+      <c r="N56" s="89"/>
+      <c r="O56" s="89"/>
+      <c r="P56" s="89"/>
+      <c r="Q56" s="89"/>
+      <c r="R56" s="89"/>
+      <c r="S56" s="90"/>
     </row>
     <row r="57" spans="1:26" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="58"/>
       <c r="S57" s="57"/>
     </row>
     <row r="58" spans="1:26" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="193" t="s">
+      <c r="A58" s="91" t="s">
         <v>90</v>
       </c>
-      <c r="B58" s="194"/>
-      <c r="C58" s="194"/>
-      <c r="D58" s="194"/>
-      <c r="E58" s="194"/>
-      <c r="F58" s="194"/>
-      <c r="G58" s="194"/>
-      <c r="H58" s="194"/>
-      <c r="I58" s="194"/>
-      <c r="J58" s="194"/>
-      <c r="K58" s="194"/>
-      <c r="L58" s="194"/>
-      <c r="M58" s="194"/>
-      <c r="N58" s="194"/>
-      <c r="O58" s="194"/>
-      <c r="P58" s="194"/>
-      <c r="Q58" s="194"/>
-      <c r="R58" s="194"/>
-      <c r="S58" s="195"/>
+      <c r="B58" s="92"/>
+      <c r="C58" s="92"/>
+      <c r="D58" s="92"/>
+      <c r="E58" s="92"/>
+      <c r="F58" s="92"/>
+      <c r="G58" s="92"/>
+      <c r="H58" s="92"/>
+      <c r="I58" s="92"/>
+      <c r="J58" s="92"/>
+      <c r="K58" s="92"/>
+      <c r="L58" s="92"/>
+      <c r="M58" s="92"/>
+      <c r="N58" s="92"/>
+      <c r="O58" s="92"/>
+      <c r="P58" s="92"/>
+      <c r="Q58" s="92"/>
+      <c r="R58" s="92"/>
+      <c r="S58" s="93"/>
     </row>
     <row r="59" spans="1:26" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="58"/>
@@ -3424,50 +3429,50 @@
       <c r="S60" s="57"/>
     </row>
     <row r="61" spans="1:26" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="123" t="s">
+      <c r="A61" s="88" t="s">
         <v>91</v>
       </c>
-      <c r="B61" s="124"/>
-      <c r="C61" s="124"/>
-      <c r="D61" s="124"/>
-      <c r="E61" s="124"/>
-      <c r="F61" s="124"/>
-      <c r="G61" s="124"/>
-      <c r="H61" s="124"/>
-      <c r="I61" s="124"/>
-      <c r="J61" s="124"/>
-      <c r="K61" s="124"/>
-      <c r="L61" s="124"/>
-      <c r="M61" s="124"/>
-      <c r="N61" s="124"/>
-      <c r="O61" s="124"/>
-      <c r="P61" s="124"/>
-      <c r="Q61" s="124"/>
-      <c r="R61" s="124"/>
-      <c r="S61" s="125"/>
+      <c r="B61" s="89"/>
+      <c r="C61" s="89"/>
+      <c r="D61" s="89"/>
+      <c r="E61" s="89"/>
+      <c r="F61" s="89"/>
+      <c r="G61" s="89"/>
+      <c r="H61" s="89"/>
+      <c r="I61" s="89"/>
+      <c r="J61" s="89"/>
+      <c r="K61" s="89"/>
+      <c r="L61" s="89"/>
+      <c r="M61" s="89"/>
+      <c r="N61" s="89"/>
+      <c r="O61" s="89"/>
+      <c r="P61" s="89"/>
+      <c r="Q61" s="89"/>
+      <c r="R61" s="89"/>
+      <c r="S61" s="90"/>
     </row>
     <row r="62" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="196" t="s">
+      <c r="A62" s="94" t="s">
         <v>92</v>
       </c>
-      <c r="B62" s="197"/>
-      <c r="C62" s="197"/>
-      <c r="D62" s="197"/>
-      <c r="E62" s="197"/>
-      <c r="F62" s="197"/>
-      <c r="G62" s="197"/>
-      <c r="H62" s="197"/>
-      <c r="I62" s="197"/>
-      <c r="J62" s="197"/>
-      <c r="K62" s="197"/>
-      <c r="L62" s="197"/>
-      <c r="M62" s="197"/>
-      <c r="N62" s="197"/>
-      <c r="O62" s="197"/>
-      <c r="P62" s="197"/>
-      <c r="Q62" s="197"/>
-      <c r="R62" s="197"/>
-      <c r="S62" s="198"/>
+      <c r="B62" s="95"/>
+      <c r="C62" s="95"/>
+      <c r="D62" s="95"/>
+      <c r="E62" s="95"/>
+      <c r="F62" s="95"/>
+      <c r="G62" s="95"/>
+      <c r="H62" s="95"/>
+      <c r="I62" s="95"/>
+      <c r="J62" s="95"/>
+      <c r="K62" s="95"/>
+      <c r="L62" s="95"/>
+      <c r="M62" s="95"/>
+      <c r="N62" s="95"/>
+      <c r="O62" s="95"/>
+      <c r="P62" s="95"/>
+      <c r="Q62" s="95"/>
+      <c r="R62" s="95"/>
+      <c r="S62" s="96"/>
       <c r="W62" s="59"/>
       <c r="X62" s="59"/>
       <c r="Y62" s="59"/>
@@ -3504,12 +3509,12 @@
     </row>
     <row r="65" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="58"/>
-      <c r="J65" s="199" t="s">
+      <c r="J65" s="73" t="s">
         <v>93</v>
       </c>
-      <c r="K65" s="199"/>
-      <c r="L65" s="199"/>
-      <c r="M65" s="199"/>
+      <c r="K65" s="73"/>
+      <c r="L65" s="73"/>
+      <c r="M65" s="73"/>
       <c r="N65" s="64"/>
       <c r="O65" s="64"/>
       <c r="S65" s="57"/>
@@ -3541,11 +3546,11 @@
     <row r="68" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="58"/>
       <c r="H68" s="67"/>
-      <c r="J68" s="199" t="s">
-        <v>96</v>
-      </c>
-      <c r="K68" s="199"/>
-      <c r="L68" s="199"/>
+      <c r="J68" s="205" t="s">
+        <v>98</v>
+      </c>
+      <c r="K68" s="205"/>
+      <c r="L68" s="205"/>
       <c r="M68" s="67"/>
       <c r="N68" s="64"/>
       <c r="O68" s="67"/>
@@ -3574,27 +3579,27 @@
       <c r="S69" s="54"/>
     </row>
     <row r="70" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="200" t="s">
-        <v>97</v>
-      </c>
-      <c r="B70" s="201"/>
-      <c r="C70" s="201"/>
-      <c r="D70" s="201"/>
-      <c r="E70" s="201"/>
-      <c r="F70" s="201"/>
-      <c r="G70" s="201"/>
-      <c r="H70" s="201"/>
-      <c r="I70" s="201"/>
-      <c r="J70" s="201"/>
-      <c r="K70" s="201"/>
-      <c r="L70" s="201"/>
-      <c r="M70" s="201"/>
-      <c r="N70" s="201"/>
-      <c r="O70" s="201"/>
-      <c r="P70" s="201"/>
-      <c r="Q70" s="201"/>
-      <c r="R70" s="201"/>
-      <c r="S70" s="202"/>
+      <c r="A70" s="74" t="s">
+        <v>96</v>
+      </c>
+      <c r="B70" s="75"/>
+      <c r="C70" s="75"/>
+      <c r="D70" s="75"/>
+      <c r="E70" s="75"/>
+      <c r="F70" s="75"/>
+      <c r="G70" s="75"/>
+      <c r="H70" s="75"/>
+      <c r="I70" s="75"/>
+      <c r="J70" s="75"/>
+      <c r="K70" s="75"/>
+      <c r="L70" s="75"/>
+      <c r="M70" s="75"/>
+      <c r="N70" s="75"/>
+      <c r="O70" s="75"/>
+      <c r="P70" s="75"/>
+      <c r="Q70" s="75"/>
+      <c r="R70" s="75"/>
+      <c r="S70" s="76"/>
     </row>
     <row r="71" spans="1:19" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="61"/>
@@ -3619,25 +3624,25 @@
     </row>
     <row r="72" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="63"/>
-      <c r="I72" s="203"/>
-      <c r="J72" s="203"/>
-      <c r="K72" s="203"/>
-      <c r="L72" s="203"/>
-      <c r="M72" s="203"/>
+      <c r="I72" s="77"/>
+      <c r="J72" s="77"/>
+      <c r="K72" s="77"/>
+      <c r="L72" s="77"/>
+      <c r="M72" s="77"/>
       <c r="S72" s="57"/>
     </row>
     <row r="73" spans="1:19" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="58"/>
-      <c r="D73" s="199"/>
-      <c r="E73" s="199"/>
-      <c r="F73" s="199"/>
-      <c r="G73" s="199"/>
-      <c r="J73" s="199" t="s">
+      <c r="D73" s="73"/>
+      <c r="E73" s="73"/>
+      <c r="F73" s="73"/>
+      <c r="G73" s="73"/>
+      <c r="J73" s="73" t="s">
         <v>93</v>
       </c>
-      <c r="K73" s="199"/>
-      <c r="L73" s="199"/>
-      <c r="M73" s="199"/>
+      <c r="K73" s="73"/>
+      <c r="L73" s="73"/>
+      <c r="M73" s="73"/>
       <c r="S73" s="57"/>
     </row>
     <row r="74" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3647,12 +3652,12 @@
       <c r="F74" s="66"/>
       <c r="G74" s="66"/>
       <c r="J74" s="65" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L74" s="65"/>
-      <c r="M74" s="204"/>
-      <c r="N74" s="204"/>
-      <c r="O74" s="204"/>
+      <c r="M74" s="78"/>
+      <c r="N74" s="78"/>
+      <c r="O74" s="78"/>
       <c r="S74" s="57"/>
     </row>
     <row r="75" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3665,30 +3670,30 @@
         <v>95</v>
       </c>
       <c r="L75" s="65"/>
-      <c r="M75" s="204"/>
-      <c r="N75" s="204"/>
-      <c r="O75" s="204"/>
+      <c r="M75" s="78"/>
+      <c r="N75" s="78"/>
+      <c r="O75" s="78"/>
       <c r="S75" s="57"/>
     </row>
     <row r="76" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="58"/>
-      <c r="D76" s="199"/>
-      <c r="E76" s="199"/>
-      <c r="F76" s="199"/>
+      <c r="D76" s="73"/>
+      <c r="E76" s="73"/>
+      <c r="F76" s="73"/>
       <c r="G76" s="67"/>
       <c r="H76" s="67"/>
-      <c r="J76" s="199" t="s">
-        <v>96</v>
-      </c>
-      <c r="K76" s="199"/>
-      <c r="L76" s="199"/>
+      <c r="J76" s="205" t="s">
+        <v>99</v>
+      </c>
+      <c r="K76" s="205"/>
+      <c r="L76" s="205"/>
       <c r="M76" s="65"/>
       <c r="N76" s="65"/>
-      <c r="O76" s="204"/>
-      <c r="P76" s="204"/>
+      <c r="O76" s="78"/>
+      <c r="P76" s="78"/>
       <c r="S76" s="57"/>
     </row>
-    <row r="77" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="70"/>
       <c r="B77" s="71"/>
       <c r="C77" s="71"/>
@@ -3711,110 +3716,6 @@
     </row>
   </sheetData>
   <mergeCells count="118">
-    <mergeCell ref="J68:L68"/>
-    <mergeCell ref="A70:S70"/>
-    <mergeCell ref="I72:M72"/>
-    <mergeCell ref="D73:G73"/>
-    <mergeCell ref="J73:M73"/>
-    <mergeCell ref="M74:O74"/>
-    <mergeCell ref="M75:O75"/>
-    <mergeCell ref="D76:F76"/>
-    <mergeCell ref="J76:L76"/>
-    <mergeCell ref="O76:P76"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="E53:J53"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="E54:J54"/>
-    <mergeCell ref="A56:S56"/>
-    <mergeCell ref="A58:S58"/>
-    <mergeCell ref="A61:S61"/>
-    <mergeCell ref="A62:S62"/>
-    <mergeCell ref="J65:M65"/>
-    <mergeCell ref="A48:J48"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="E49:J49"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="E50:J50"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="E51:J51"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="E52:J52"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="G46:I46"/>
-    <mergeCell ref="K46:M46"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="P46:S46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="K47:M47"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="P47:S47"/>
-    <mergeCell ref="A41:F41"/>
-    <mergeCell ref="G41:J41"/>
-    <mergeCell ref="K41:N41"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="G42:J42"/>
-    <mergeCell ref="K42:N42"/>
-    <mergeCell ref="A44:S44"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="K45:M45"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="P45:S45"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="G38:J38"/>
-    <mergeCell ref="K38:N38"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="G39:J39"/>
-    <mergeCell ref="K39:N39"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="G40:J40"/>
-    <mergeCell ref="K40:N40"/>
-    <mergeCell ref="A19:S19"/>
-    <mergeCell ref="A20:S20"/>
-    <mergeCell ref="A21:S21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="A34:O35"/>
-    <mergeCell ref="G36:J36"/>
-    <mergeCell ref="K36:N36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="G37:J37"/>
-    <mergeCell ref="K37:N37"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="Q15:S15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="O16:Q16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="Q17:S17"/>
-    <mergeCell ref="O11:S11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:S12"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="O13:Q13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G14:J14"/>
-    <mergeCell ref="K14:M14"/>
-    <mergeCell ref="N14:P14"/>
-    <mergeCell ref="Q14:S14"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="I11:L11"/>
-    <mergeCell ref="M11:N11"/>
     <mergeCell ref="A2:C5"/>
     <mergeCell ref="D2:P5"/>
     <mergeCell ref="Q2:S5"/>
@@ -3829,6 +3730,110 @@
     <mergeCell ref="I9:L9"/>
     <mergeCell ref="M9:O9"/>
     <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:L11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="O11:S11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:S12"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="O13:Q13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:J14"/>
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="N14:P14"/>
+    <mergeCell ref="Q14:S14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="Q15:S15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="O16:Q16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="Q17:S17"/>
+    <mergeCell ref="A19:S19"/>
+    <mergeCell ref="A20:S20"/>
+    <mergeCell ref="A21:S21"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="A34:O35"/>
+    <mergeCell ref="G36:J36"/>
+    <mergeCell ref="K36:N36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="K37:N37"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="G38:J38"/>
+    <mergeCell ref="K38:N38"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="G39:J39"/>
+    <mergeCell ref="K39:N39"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="G40:J40"/>
+    <mergeCell ref="K40:N40"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="G41:J41"/>
+    <mergeCell ref="K41:N41"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="G42:J42"/>
+    <mergeCell ref="K42:N42"/>
+    <mergeCell ref="A44:S44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="K45:M45"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="P45:S45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="K46:M46"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="P46:S46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="P47:S47"/>
+    <mergeCell ref="A48:J48"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="E49:J49"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="E50:J50"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="E51:J51"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="E52:J52"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="E53:J53"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="E54:J54"/>
+    <mergeCell ref="A56:S56"/>
+    <mergeCell ref="A58:S58"/>
+    <mergeCell ref="A61:S61"/>
+    <mergeCell ref="A62:S62"/>
+    <mergeCell ref="J65:M65"/>
+    <mergeCell ref="J68:L68"/>
+    <mergeCell ref="A70:S70"/>
+    <mergeCell ref="I72:M72"/>
+    <mergeCell ref="D73:G73"/>
+    <mergeCell ref="J73:M73"/>
+    <mergeCell ref="M74:O74"/>
+    <mergeCell ref="M75:O75"/>
+    <mergeCell ref="D76:F76"/>
+    <mergeCell ref="J76:L76"/>
+    <mergeCell ref="O76:P76"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B23:B33" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>